<commit_message>
Added functions convert_dates, is_excel_date, get_code_choice. Updated date_to_jul. Moved conversion funtions to convert.R. Added globals.R. Fixed file path issue
</commit_message>
<xml_diff>
--- a/files/Templates/collected_data.xlsx
+++ b/files/Templates/collected_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpo\Documents\Research\STICS\Code\mkSTICSfiles\files\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpo\Documents\Research\STICS\Code\mkSTICSfiles\files\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8435BD-6E33-4294-89A4-E4A9A779B45D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424D330F-59F3-4D69-84F8-7B0E19D330F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="30936" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="management" sheetId="8" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="stations" sheetId="6" r:id="rId3"/>
     <sheet name="usms" sheetId="1" r:id="rId4"/>
     <sheet name="observations" sheetId="9" r:id="rId5"/>
-    <sheet name="options" sheetId="4" state="hidden" r:id="rId6"/>
+    <sheet name="options" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Fertilizer_Application">Table3[Fertilizer_Application]</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="178">
   <si>
     <t>usm_name</t>
   </si>
@@ -421,9 +421,6 @@
     <t>amount_15</t>
   </si>
   <si>
-    <t>irrigation_date_16</t>
-  </si>
-  <si>
     <t>Irrigation</t>
   </si>
   <si>
@@ -557,6 +554,36 @@
   </si>
   <si>
     <t>albedo</t>
+  </si>
+  <si>
+    <t>harvest_end</t>
+  </si>
+  <si>
+    <t>harvest_date2</t>
+  </si>
+  <si>
+    <t>automatic_irr_depth</t>
+  </si>
+  <si>
+    <t>harvest</t>
+  </si>
+  <si>
+    <t>irrigation_type</t>
+  </si>
+  <si>
+    <t>irr_efficiency</t>
+  </si>
+  <si>
+    <t>Irrigation Location</t>
+  </si>
+  <si>
+    <t>1 = above the foliage</t>
+  </si>
+  <si>
+    <t>2 = below the foliage above the soil</t>
+  </si>
+  <si>
+    <t>3 = in the soil</t>
   </si>
 </sst>
 </file>
@@ -601,7 +628,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,6 +785,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="gray0625">
+        <fgColor theme="0" tint="-0.14993743705557422"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="14">
     <border>
@@ -908,7 +941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -962,6 +995,10 @@
     <xf numFmtId="0" fontId="3" fillId="26" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -989,122 +1026,30 @@
     <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="55">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -1166,76 +1111,6 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray0625">
-          <fgColor theme="0" tint="-0.24994659260841701"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1565,6 +1440,171 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray0625">
+          <fgColor theme="0" tint="-0.24994659260841701"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1591,24 +1631,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}" name="Table6" displayName="Table6" ref="A2:AT100" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7">
-  <autoFilter ref="A2:AT100" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}"/>
-  <tableColumns count="46">
-    <tableColumn id="1" xr3:uid="{6B129591-A0EC-4CC8-AA8E-70259B5C9131}" name="file_name" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{1FBFF361-0229-404E-A60E-FCEC995B36AD}" name="year" dataDxfId="4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}" name="Table6" displayName="Table6" ref="A2:AX100" totalsRowShown="0" headerRowDxfId="48" headerRowBorderDxfId="47" tableBorderDxfId="46">
+  <autoFilter ref="A2:AX100" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}"/>
+  <tableColumns count="50">
+    <tableColumn id="1" xr3:uid="{6B129591-A0EC-4CC8-AA8E-70259B5C9131}" name="file_name" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{1FBFF361-0229-404E-A60E-FCEC995B36AD}" name="year" dataDxfId="44"/>
     <tableColumn id="3" xr3:uid="{416116E5-319A-4096-B7E5-AF8ADEF0E80A}" name="tillage_date"/>
-    <tableColumn id="4" xr3:uid="{781FB9F7-258C-4E50-8A90-CAA110FA989E}" name="tillage_depth" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{781FB9F7-258C-4E50-8A90-CAA110FA989E}" name="tillage_depth" dataDxfId="43"/>
     <tableColumn id="5" xr3:uid="{A768ED69-1CCB-4A41-99C1-D5042177408B}" name="planting_date"/>
     <tableColumn id="6" xr3:uid="{5517C570-4D1C-46EC-9FB0-4FEA929440E1}" name="planting_depth"/>
-    <tableColumn id="7" xr3:uid="{8F3D9EFB-6197-44D6-9CAB-532096E5D0DE}" name="plants_per_m2" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{8F3D9EFB-6197-44D6-9CAB-532096E5D0DE}" name="plants_per_m2" dataDxfId="42"/>
     <tableColumn id="8" xr3:uid="{7DEB259C-DAE3-4A1E-B476-951FEF30ABD2}" name="emergence"/>
     <tableColumn id="9" xr3:uid="{8590CC43-CF1F-45A9-A612-CE3749B53C84}" name="flowering"/>
-    <tableColumn id="10" xr3:uid="{DAF1F67C-7CB4-4AD2-B1D4-24884C7C9D57}" name="maturity" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{DAF1F67C-7CB4-4AD2-B1D4-24884C7C9D57}" name="maturity" dataDxfId="41"/>
     <tableColumn id="11" xr3:uid="{1651DE3B-149A-4121-AFB0-BA33E8308050}" name="application_date"/>
     <tableColumn id="12" xr3:uid="{358B23A5-F859-4B79-9182-F98F3D69F461}" name="kg_N_per_ha"/>
     <tableColumn id="13" xr3:uid="{FEB67719-45D9-4389-A438-548C552EBED6}" name="fert_type"/>
     <tableColumn id="14" xr3:uid="{B9B3005C-6E63-4AA3-BE8E-646D9659B76F}" name="fert_location"/>
-    <tableColumn id="15" xr3:uid="{F5737449-F543-4637-B8F3-6DBD1B98EDA2}" name="fert_depth" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{F5737449-F543-4637-B8F3-6DBD1B98EDA2}" name="fert_depth" dataDxfId="40"/>
+    <tableColumn id="49" xr3:uid="{1DACF6E4-1D01-4D98-B61F-06AED8D28283}" name="irrigation_type"/>
+    <tableColumn id="48" xr3:uid="{E053F1CC-2741-44D0-BCB6-E2638B921A91}" name="irr_efficiency"/>
     <tableColumn id="16" xr3:uid="{AA12C7D8-D645-4337-B05C-CB5F5C197AE4}" name="irrigation_date_1"/>
     <tableColumn id="17" xr3:uid="{017BC113-D478-4E04-AEE6-020CA6B48738}" name="amount_1"/>
     <tableColumn id="18" xr3:uid="{498ED556-89DC-49A5-A6C1-DF741DBED2EF}" name="irrigation_date_2"/>
@@ -1639,7 +1681,9 @@
     <tableColumn id="43" xr3:uid="{0A0B6CAB-9EC9-4492-A667-1846AE54A020}" name="amount_14"/>
     <tableColumn id="44" xr3:uid="{7DD1FA19-1C12-4443-9EB3-267851A488BA}" name="irrigation_date_15"/>
     <tableColumn id="45" xr3:uid="{A69E1720-4BA7-4736-9E85-A0E33013B090}" name="amount_15"/>
-    <tableColumn id="46" xr3:uid="{A0DFD622-ADA5-48E2-B689-A17242FFBEEA}" name="irrigation_date_16"/>
+    <tableColumn id="51" xr3:uid="{D644A008-911D-42DE-B5AE-3D97E8D9CBE3}" name="automatic_irr_depth"/>
+    <tableColumn id="47" xr3:uid="{8142D301-45D6-476E-91F5-4C775D8382CE}" name="harvest_date2"/>
+    <tableColumn id="50" xr3:uid="{A3119A2B-1FF4-4688-A8C7-EA84F5130A56}" name="harvest_end"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1655,11 +1699,21 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{EC7F3CD2-B7DD-4AB9-A1D1-61C6B8E31CF2}" name="Table11" displayName="Table11" ref="K1:K4" totalsRowShown="0">
+  <autoFilter ref="K1:K4" xr:uid="{EC7F3CD2-B7DD-4AB9-A1D1-61C6B8E31CF2}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{684BC5C4-FC4C-4A03-9843-BEAD87C7E594}" name="Irrigation Location"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}" name="Table7" displayName="Table7" ref="A2:BS100" totalsRowShown="0" headerRowDxfId="54" headerRowBorderDxfId="53" tableBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}" name="Table7" displayName="Table7" ref="A2:BS100" totalsRowShown="0" headerRowDxfId="39" headerRowBorderDxfId="38" tableBorderDxfId="37">
   <autoFilter ref="A2:BS100" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}"/>
   <tableColumns count="71">
-    <tableColumn id="1" xr3:uid="{4674EE1C-2CD4-485E-8B27-A14DEFFAAD8A}" name="soil_profile_name" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{4674EE1C-2CD4-485E-8B27-A14DEFFAAD8A}" name="soil_profile_name" dataDxfId="36"/>
     <tableColumn id="2" xr3:uid="{72D785FE-A1AF-4E08-AB14-39FAD15DB9BD}" name="thickness_1"/>
     <tableColumn id="3" xr3:uid="{1838D7E8-2B3C-471C-9A0B-D70D91F18417}" name="pH"/>
     <tableColumn id="71" xr3:uid="{931F79EB-F524-439C-8A88-ED674075FA7F}" name="albedo"/>
@@ -1671,110 +1725,110 @@
     <tableColumn id="40" xr3:uid="{EC836542-6DD7-49C9-82D9-B724BCE18341}" name="SON_1"/>
     <tableColumn id="41" xr3:uid="{F7750E58-5B0E-4494-87AF-B025671824DE}" name="CN_ratio"/>
     <tableColumn id="8" xr3:uid="{0592115C-328E-42C4-B9CB-D43026D4FC27}" name="FC_1"/>
-    <tableColumn id="42" xr3:uid="{5C21A417-1737-43F1-BC15-EC087A009A68}" name="FC_1_unit" dataDxfId="50"/>
+    <tableColumn id="42" xr3:uid="{5C21A417-1737-43F1-BC15-EC087A009A68}" name="FC_1_unit" dataDxfId="35"/>
     <tableColumn id="9" xr3:uid="{C1383A59-387E-4667-852A-B0CF467088F3}" name="WP_1"/>
-    <tableColumn id="43" xr3:uid="{75E60C07-9873-41B6-AB5A-253087B95CFA}" name="WP_1_unit" dataDxfId="49"/>
+    <tableColumn id="43" xr3:uid="{75E60C07-9873-41B6-AB5A-253087B95CFA}" name="WP_1_unit" dataDxfId="34"/>
     <tableColumn id="10" xr3:uid="{34D0D911-5DB4-457F-88A7-76A42B57EE1A}" name="initial_NO3_1"/>
-    <tableColumn id="52" xr3:uid="{630D852C-736F-4D0D-8BB3-6EB32B59A383}" name="initial_NO3_1_units" dataDxfId="48"/>
+    <tableColumn id="52" xr3:uid="{630D852C-736F-4D0D-8BB3-6EB32B59A383}" name="initial_NO3_1_units" dataDxfId="33"/>
     <tableColumn id="53" xr3:uid="{CEF78893-60AA-4A20-A771-E76562B8EBC1}" name="initial_NH4_1"/>
-    <tableColumn id="11" xr3:uid="{58B6280A-10C4-4120-9FF8-93150CE70C6B}" name="initial_NH4_1_units" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{58B6280A-10C4-4120-9FF8-93150CE70C6B}" name="initial_NH4_1_units" dataDxfId="32"/>
     <tableColumn id="12" xr3:uid="{FD043EB5-2678-4920-8D76-EBE8316E27AA}" name="thickness_2"/>
     <tableColumn id="13" xr3:uid="{F124AE04-B447-4F21-A0E8-7B26199C0F49}" name="%_sand_2"/>
     <tableColumn id="14" xr3:uid="{F119498A-3A35-40E3-A753-7CF13D724118}" name="%_clay_2"/>
     <tableColumn id="15" xr3:uid="{AE51522F-6903-42D4-88CE-A95BCE8C77EF}" name="BD_2"/>
     <tableColumn id="16" xr3:uid="{12076489-6AD7-4297-A729-20EF93AEE58D}" name="SOC_2"/>
     <tableColumn id="17" xr3:uid="{D6D5EFD4-69CC-4AF2-8C6B-0B430468C4C2}" name="FC_2"/>
-    <tableColumn id="44" xr3:uid="{7158FD96-C69C-40D1-A3B8-2D043DF66D42}" name="FC_2_unit" dataDxfId="46"/>
+    <tableColumn id="44" xr3:uid="{7158FD96-C69C-40D1-A3B8-2D043DF66D42}" name="FC_2_unit" dataDxfId="31"/>
     <tableColumn id="18" xr3:uid="{BBF6A61D-2092-4DF7-8C38-9024164291AE}" name="WP_2"/>
-    <tableColumn id="45" xr3:uid="{2A662E87-2699-41FA-AF9F-C807E1C2112B}" name="WP_2_unit" dataDxfId="45"/>
+    <tableColumn id="45" xr3:uid="{2A662E87-2699-41FA-AF9F-C807E1C2112B}" name="WP_2_unit" dataDxfId="30"/>
     <tableColumn id="19" xr3:uid="{BB4B796C-CA3E-424C-87B0-4BF33581B61B}" name="initial_NO3_2"/>
-    <tableColumn id="54" xr3:uid="{13CDB225-A28A-424D-943F-330A6ABE0CF2}" name="initial_NO3_2_unit" dataDxfId="44"/>
+    <tableColumn id="54" xr3:uid="{13CDB225-A28A-424D-943F-330A6ABE0CF2}" name="initial_NO3_2_unit" dataDxfId="29"/>
     <tableColumn id="55" xr3:uid="{333E59C3-3A13-4C92-9169-AC90D5E5D3EB}" name="initial_NH4_2"/>
-    <tableColumn id="20" xr3:uid="{613F6ECB-AFEC-4E8A-BD78-2579E90B1783}" name="initial_NH4_2_unit" dataDxfId="43"/>
-    <tableColumn id="21" xr3:uid="{5D7B3549-7F90-410E-90FF-149F4376EBB7}" name="thickness_3" dataDxfId="42"/>
+    <tableColumn id="20" xr3:uid="{613F6ECB-AFEC-4E8A-BD78-2579E90B1783}" name="initial_NH4_2_unit" dataDxfId="28"/>
+    <tableColumn id="21" xr3:uid="{5D7B3549-7F90-410E-90FF-149F4376EBB7}" name="thickness_3" dataDxfId="27"/>
     <tableColumn id="22" xr3:uid="{6C917DE4-8D95-496E-A6F1-EAB7450774EE}" name="%_sand_3"/>
     <tableColumn id="23" xr3:uid="{90DE7FE2-3A23-4294-8BD0-2D321FF71179}" name="%_clay_3"/>
     <tableColumn id="24" xr3:uid="{C874CBBB-CB06-4239-AE9B-72564A3EDC14}" name="BD_3"/>
     <tableColumn id="25" xr3:uid="{49CED3FB-E83C-4973-A99D-DAC6B3AFC7B1}" name="SOC_3"/>
     <tableColumn id="26" xr3:uid="{63FB3901-EBED-4379-9E9C-83064A8ADD01}" name="FC_3"/>
-    <tableColumn id="47" xr3:uid="{5C201AAC-779E-4362-9603-51762D2AD5CF}" name="FC_3_unit" dataDxfId="41"/>
+    <tableColumn id="47" xr3:uid="{5C201AAC-779E-4362-9603-51762D2AD5CF}" name="FC_3_unit" dataDxfId="26"/>
     <tableColumn id="27" xr3:uid="{6EEACF0E-3934-49DF-9991-42C2DB718BE0}" name="WP_3"/>
-    <tableColumn id="48" xr3:uid="{67EEF171-24DC-4B50-B1F4-746B04E8F368}" name="WP_3_unit" dataDxfId="40"/>
+    <tableColumn id="48" xr3:uid="{67EEF171-24DC-4B50-B1F4-746B04E8F368}" name="WP_3_unit" dataDxfId="25"/>
     <tableColumn id="28" xr3:uid="{7AAE3F1E-C60E-4E11-A023-F09548D5AA39}" name="initial_NO3_3"/>
-    <tableColumn id="56" xr3:uid="{2B23B0A6-3617-432B-8EEA-E2AC0892F317}" name="initial_NO3_3_unit" dataDxfId="39"/>
+    <tableColumn id="56" xr3:uid="{2B23B0A6-3617-432B-8EEA-E2AC0892F317}" name="initial_NO3_3_unit" dataDxfId="24"/>
     <tableColumn id="57" xr3:uid="{1D0A3587-38DB-4073-B5D4-36DA82425955}" name="initial_NH4_3"/>
-    <tableColumn id="29" xr3:uid="{4BF74EC8-B9F2-42F0-AA7F-7CF70391A1FD}" name="initial_NH4_3_unit" dataDxfId="38"/>
-    <tableColumn id="30" xr3:uid="{4F55D6E9-95FD-4FC3-8012-EBB0DDAD9C3D}" name="thickness_4" dataDxfId="37"/>
+    <tableColumn id="29" xr3:uid="{4BF74EC8-B9F2-42F0-AA7F-7CF70391A1FD}" name="initial_NH4_3_unit" dataDxfId="23"/>
+    <tableColumn id="30" xr3:uid="{4F55D6E9-95FD-4FC3-8012-EBB0DDAD9C3D}" name="thickness_4" dataDxfId="22"/>
     <tableColumn id="31" xr3:uid="{4C1178FA-055B-4F19-A181-638D37A24EB6}" name="%_sand_4"/>
     <tableColumn id="32" xr3:uid="{7BBFA3FD-BBE5-4B68-A551-EFDEA7062540}" name="%_clay_4"/>
     <tableColumn id="33" xr3:uid="{D0607A27-FB9E-4DA9-A7F3-7A932B2608A4}" name="BD_4"/>
     <tableColumn id="34" xr3:uid="{BD46131F-AB56-411A-8742-B77FBBE1967B}" name="SOC_4"/>
     <tableColumn id="35" xr3:uid="{EC2EEDB8-3CC6-4DEE-9309-DBA3B11A2D16}" name="FC_4"/>
-    <tableColumn id="50" xr3:uid="{D1D16E63-48A7-4CF1-950A-55FD748CC035}" name="FC_4_unit" dataDxfId="36"/>
-    <tableColumn id="36" xr3:uid="{2FE3E094-F831-4B6A-8F68-958367A1890E}" name="WP_4" dataDxfId="35"/>
-    <tableColumn id="51" xr3:uid="{FDA92DA7-3473-43EC-9CF7-2973FA9CC4D4}" name="WP_4_unit" dataDxfId="34"/>
-    <tableColumn id="58" xr3:uid="{BE460051-3822-4F7B-9128-B9FF3E679D50}" name="initial_NO3_4" dataDxfId="33"/>
-    <tableColumn id="37" xr3:uid="{8064862C-F8DC-4543-B5CF-D282DD564B1D}" name="initial_NO3_4_unit" dataDxfId="32"/>
-    <tableColumn id="59" xr3:uid="{17C5A0C3-B5F4-4AAB-876C-FC876098B9C8}" name="initial_NH4_4" dataDxfId="31"/>
-    <tableColumn id="38" xr3:uid="{251884D5-BA16-4F6E-89D1-06011C0ABD02}" name="initial_NH4_4_unit" dataDxfId="30"/>
+    <tableColumn id="50" xr3:uid="{D1D16E63-48A7-4CF1-950A-55FD748CC035}" name="FC_4_unit" dataDxfId="21"/>
+    <tableColumn id="36" xr3:uid="{2FE3E094-F831-4B6A-8F68-958367A1890E}" name="WP_4" dataDxfId="20"/>
+    <tableColumn id="51" xr3:uid="{FDA92DA7-3473-43EC-9CF7-2973FA9CC4D4}" name="WP_4_unit" dataDxfId="19"/>
+    <tableColumn id="58" xr3:uid="{BE460051-3822-4F7B-9128-B9FF3E679D50}" name="initial_NO3_4" dataDxfId="18"/>
+    <tableColumn id="37" xr3:uid="{8064862C-F8DC-4543-B5CF-D282DD564B1D}" name="initial_NO3_4_unit" dataDxfId="17"/>
+    <tableColumn id="59" xr3:uid="{17C5A0C3-B5F4-4AAB-876C-FC876098B9C8}" name="initial_NH4_4" dataDxfId="16"/>
+    <tableColumn id="38" xr3:uid="{251884D5-BA16-4F6E-89D1-06011C0ABD02}" name="initial_NH4_4_unit" dataDxfId="15"/>
     <tableColumn id="46" xr3:uid="{5545ADBB-3E57-4FCE-9979-330500D810A6}" name="thickness_5"/>
     <tableColumn id="49" xr3:uid="{28F4610E-A232-42D7-866E-B72AB5FC38D8}" name="%_sand_5"/>
     <tableColumn id="60" xr3:uid="{9557F7B0-0944-4CA4-8B86-630B4073480C}" name="%_clay_5"/>
     <tableColumn id="61" xr3:uid="{6977D0A0-E571-46FB-8186-DF22D992C4B6}" name="BD_5"/>
     <tableColumn id="62" xr3:uid="{762BF513-B3A9-4714-B788-A74D32CD414B}" name="SOC_5"/>
     <tableColumn id="63" xr3:uid="{F840DA58-F957-445A-8704-4823DC13AEC7}" name="FC_5"/>
-    <tableColumn id="64" xr3:uid="{47AF2E86-82B6-4018-9B34-1B9AA21CC4AF}" name="FC_5_unit" dataDxfId="29"/>
+    <tableColumn id="64" xr3:uid="{47AF2E86-82B6-4018-9B34-1B9AA21CC4AF}" name="FC_5_unit" dataDxfId="14"/>
     <tableColumn id="65" xr3:uid="{73133DDD-77CC-4B8F-AF63-0B5537B95DE3}" name="WP_5"/>
-    <tableColumn id="66" xr3:uid="{7CB1FDF0-326D-4446-9AAC-1DB26A38AAB4}" name="WP_5_unit" dataDxfId="28"/>
+    <tableColumn id="66" xr3:uid="{7CB1FDF0-326D-4446-9AAC-1DB26A38AAB4}" name="WP_5_unit" dataDxfId="13"/>
     <tableColumn id="67" xr3:uid="{AF697735-FE14-47A1-8029-532D47D2E5C7}" name="initial_NO3_5"/>
-    <tableColumn id="68" xr3:uid="{B9420E91-6BD4-467A-B4C2-A6E2DEAE7AC0}" name="initial_NO3_5_unit" dataDxfId="27"/>
-    <tableColumn id="69" xr3:uid="{FF6305CB-A38F-4242-9850-7966AD42A38B}" name="initial_NH4_5" dataDxfId="26"/>
-    <tableColumn id="70" xr3:uid="{B5EFBF0D-28C6-43EC-8EBE-8FDCF2F3F407}" name="initial_NH4_5_unit" dataDxfId="25"/>
+    <tableColumn id="68" xr3:uid="{B9420E91-6BD4-467A-B4C2-A6E2DEAE7AC0}" name="initial_NO3_5_unit" dataDxfId="12"/>
+    <tableColumn id="69" xr3:uid="{FF6305CB-A38F-4242-9850-7966AD42A38B}" name="initial_NH4_5" dataDxfId="11"/>
+    <tableColumn id="70" xr3:uid="{B5EFBF0D-28C6-43EC-8EBE-8FDCF2F3F407}" name="initial_NH4_5_unit" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}" name="Table5" displayName="Table5" ref="A1:D109" totalsRowShown="0" headerRowBorderDxfId="24" tableBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}" name="Table5" displayName="Table5" ref="A1:D109" totalsRowShown="0" headerRowBorderDxfId="54" tableBorderDxfId="53">
   <autoFilter ref="A1:D109" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9BCD565A-9AEA-41E2-A4E9-5770EC475FD6}" name="station_name" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{2FFE488A-7A94-4C6D-BFBF-9D19F7354A7D}" name="latitude" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{7A348C5F-5ECA-4DC4-9498-87CB7828B623}" name="PET_calculation" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{528CFAC7-D6A1-4BF3-A218-92AEE6E73C93}" name="average_windspeed" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{9BCD565A-9AEA-41E2-A4E9-5770EC475FD6}" name="station_name" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{2FFE488A-7A94-4C6D-BFBF-9D19F7354A7D}" name="latitude" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{7A348C5F-5ECA-4DC4-9498-87CB7828B623}" name="PET_calculation" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{528CFAC7-D6A1-4BF3-A218-92AEE6E73C93}" name="average_windspeed" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}" name="Table8" displayName="Table8" ref="A2:J100" totalsRowShown="0" headerRowBorderDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}" name="Table8" displayName="Table8" ref="A2:J100" totalsRowShown="0" headerRowBorderDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="A2:J100" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{524AE2E3-B113-41B0-849D-8331462FB910}" name="usm_name" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{524AE2E3-B113-41B0-849D-8331462FB910}" name="usm_name" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{C58B90D4-B75A-409B-9D58-E09932ABF65C}" name="simulation_start"/>
-    <tableColumn id="3" xr3:uid="{DDB99A97-7CAB-4C4A-87B0-F44791A69661}" name="simulation_end" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{CA3AF775-2448-4D7D-9193-B5BBEE39AD09}" name="management_file_name" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{DDB99A97-7CAB-4C4A-87B0-F44791A69661}" name="simulation_end" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{CA3AF775-2448-4D7D-9193-B5BBEE39AD09}" name="management_file_name" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{C4CB74A7-2660-4D67-9D08-D7802D112D6D}" name="soil_profile_name"/>
     <tableColumn id="6" xr3:uid="{EE8564A9-D685-42B6-914D-B5F77F840B11}" name="weather_station_name"/>
     <tableColumn id="7" xr3:uid="{DF70C6E4-2795-4D3D-B86B-8B48BE8FB3E1}" name="plant_file"/>
-    <tableColumn id="8" xr3:uid="{B3D6750F-E334-4A3F-A048-BA40F1D2EC0C}" name="cultivar_code" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{B3D6750F-E334-4A3F-A048-BA40F1D2EC0C}" name="cultivar_code" dataDxfId="4"/>
     <tableColumn id="9" xr3:uid="{BDB57316-D9C6-4EE3-821F-F5561E0078D9}" name="first_year"/>
-    <tableColumn id="10" xr3:uid="{733885B2-6768-4BD5-9F65-4E7F4F6262F5}" name="last_year" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{733885B2-6768-4BD5-9F65-4E7F4F6262F5}" name="last_year" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}" name="Table10" displayName="Table10" ref="A1:F30" totalsRowShown="0" headerRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}" name="Table10" displayName="Table10" ref="A1:F30" totalsRowShown="0" headerRowBorderDxfId="2">
   <autoFilter ref="A1:F30" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{F945B708-1D60-4D2B-99F2-60E35ECBDB15}" name="usm_name" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{F945B708-1D60-4D2B-99F2-60E35ECBDB15}" name="usm_name" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{A5156817-2D3F-4E14-AC57-75BA66E12293}" name="year"/>
     <tableColumn id="3" xr3:uid="{173E3383-07EB-425D-884F-01E4ECFF4626}" name="month"/>
-    <tableColumn id="4" xr3:uid="{786A5374-97E3-4942-B27A-E7E524EC0BA1}" name="day" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{786A5374-97E3-4942-B27A-E7E524EC0BA1}" name="day" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{B9B2B184-EF64-48EF-B50B-8E24249DFDCC}" name="variable 1"/>
     <tableColumn id="7" xr3:uid="{ED0F5D28-DB43-4C9B-ADB2-1706AC6D61F9}" name="variable 2"/>
   </tableColumns>
@@ -2088,7 +2142,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:AT100"/>
+  <dimension ref="A1:AX100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" style="5" customWidth="1"/>
@@ -2139,63 +2193,67 @@
     <col min="46" max="46" width="18.21875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.3">
-      <c r="C1" s="51" t="s">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C1" s="55" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="52" t="s">
+      <c r="D1" s="55"/>
+      <c r="E1" s="56" t="s">
         <v>63</v>
       </c>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="54" t="s">
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="53" t="s">
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
-      <c r="O1" s="53"/>
-      <c r="P1" s="55" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-      <c r="AD1" s="55"/>
-      <c r="AE1" s="55"/>
-      <c r="AF1" s="55"/>
-      <c r="AG1" s="55"/>
-      <c r="AH1" s="55"/>
-      <c r="AI1" s="55"/>
-      <c r="AJ1" s="55"/>
-      <c r="AK1" s="55"/>
-      <c r="AL1" s="55"/>
-      <c r="AM1" s="55"/>
-      <c r="AN1" s="55"/>
-      <c r="AO1" s="55"/>
-      <c r="AP1" s="55"/>
-      <c r="AQ1" s="55"/>
-      <c r="AR1" s="55"/>
-      <c r="AS1" s="55"/>
-      <c r="AT1" s="55"/>
-    </row>
-    <row r="2" spans="1:46" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="69" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="72"/>
+      <c r="AW1" s="70" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:50" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
         <v>52</v>
       </c>
@@ -2242,500 +2300,901 @@
         <v>62</v>
       </c>
       <c r="P2" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="R2" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="S2" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="T2" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="U2" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="V2" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="W2" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="V2" s="11" t="s">
+      <c r="X2" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="Y2" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="X2" s="11" t="s">
+      <c r="Z2" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="AA2" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="Z2" s="11" t="s">
+      <c r="AB2" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="AA2" s="11" t="s">
+      <c r="AC2" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="AB2" s="11" t="s">
+      <c r="AD2" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="AC2" s="11" t="s">
+      <c r="AE2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="AD2" s="11" t="s">
+      <c r="AF2" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="AE2" s="11" t="s">
+      <c r="AG2" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="AF2" s="11" t="s">
+      <c r="AH2" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="AG2" s="11" t="s">
+      <c r="AI2" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="AH2" s="11" t="s">
+      <c r="AJ2" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="AI2" s="11" t="s">
+      <c r="AK2" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="AJ2" s="11" t="s">
+      <c r="AL2" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="AK2" s="11" t="s">
+      <c r="AM2" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="AL2" s="11" t="s">
+      <c r="AN2" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="AM2" s="11" t="s">
+      <c r="AO2" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="AN2" s="11" t="s">
+      <c r="AP2" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="AO2" s="11" t="s">
+      <c r="AQ2" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="AP2" s="11" t="s">
+      <c r="AR2" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="AQ2" s="11" t="s">
+      <c r="AS2" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="AR2" s="11" t="s">
+      <c r="AT2" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="AS2" s="11" t="s">
+      <c r="AU2" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="AT2" s="11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.3">
-      <c r="E3" s="67"/>
+      <c r="AV2" s="71" t="s">
+        <v>170</v>
+      </c>
+      <c r="AW2" s="73" t="s">
+        <v>169</v>
+      </c>
+      <c r="AX2" s="73" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="E3" s="54"/>
       <c r="M3" s="38"/>
       <c r="N3" s="38"/>
+      <c r="P3" s="74"/>
+      <c r="Q3" s="68"/>
       <c r="AT3"/>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M4" s="38"/>
       <c r="N4" s="38"/>
-    </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P4" s="74"/>
+      <c r="Q4" s="68"/>
+      <c r="AT4"/>
+      <c r="AV4" s="68"/>
+    </row>
+    <row r="5" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M5" s="38"/>
       <c r="N5" s="38"/>
-    </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P5" s="74"/>
+      <c r="Q5" s="68"/>
+      <c r="AT5"/>
+      <c r="AV5" s="68"/>
+    </row>
+    <row r="6" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M6" s="38"/>
       <c r="N6" s="38"/>
-    </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P6" s="74"/>
+      <c r="Q6" s="68"/>
+      <c r="AT6"/>
+      <c r="AV6" s="68"/>
+    </row>
+    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M7" s="38"/>
       <c r="N7" s="38"/>
-    </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P7" s="74"/>
+      <c r="Q7" s="68"/>
+      <c r="AT7"/>
+      <c r="AV7" s="68"/>
+    </row>
+    <row r="8" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M8" s="38"/>
       <c r="N8" s="38"/>
-    </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P8" s="74"/>
+      <c r="Q8" s="68"/>
+      <c r="AT8"/>
+      <c r="AV8" s="68"/>
+    </row>
+    <row r="9" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M9" s="38"/>
       <c r="N9" s="38"/>
-    </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P9" s="74"/>
+      <c r="Q9" s="68"/>
+      <c r="AT9"/>
+      <c r="AV9" s="68"/>
+    </row>
+    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M10" s="38"/>
       <c r="N10" s="38"/>
-    </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P10" s="74"/>
+      <c r="Q10" s="68"/>
+      <c r="AT10"/>
+      <c r="AV10" s="68"/>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M11" s="38"/>
       <c r="N11" s="38"/>
-    </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P11" s="74"/>
+      <c r="Q11" s="68"/>
+      <c r="AT11"/>
+      <c r="AV11" s="68"/>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M12" s="38"/>
       <c r="N12" s="38"/>
-    </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P12" s="74"/>
+      <c r="Q12" s="68"/>
+      <c r="AT12"/>
+      <c r="AV12" s="68"/>
+    </row>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M13" s="38"/>
       <c r="N13" s="38"/>
-    </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P13" s="74"/>
+      <c r="Q13" s="68"/>
+      <c r="AT13"/>
+      <c r="AV13" s="68"/>
+    </row>
+    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M14" s="38"/>
       <c r="N14" s="38"/>
-    </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P14" s="74"/>
+      <c r="Q14" s="68"/>
+      <c r="AT14"/>
+      <c r="AV14" s="68"/>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M15" s="38"/>
       <c r="N15" s="38"/>
-    </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P15" s="74"/>
+      <c r="Q15" s="68"/>
+      <c r="AT15"/>
+      <c r="AV15" s="68"/>
+    </row>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M16" s="38"/>
       <c r="N16" s="38"/>
-    </row>
-    <row r="17" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P16" s="74"/>
+      <c r="Q16" s="68"/>
+      <c r="AT16"/>
+      <c r="AV16" s="68"/>
+    </row>
+    <row r="17" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M17" s="38"/>
       <c r="N17" s="38"/>
-    </row>
-    <row r="18" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P17" s="74"/>
+      <c r="Q17" s="68"/>
+      <c r="AT17"/>
+      <c r="AV17" s="68"/>
+    </row>
+    <row r="18" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M18" s="38"/>
       <c r="N18" s="38"/>
-    </row>
-    <row r="19" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P18" s="74"/>
+      <c r="Q18" s="68"/>
+      <c r="AT18"/>
+      <c r="AV18" s="68"/>
+    </row>
+    <row r="19" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M19" s="38"/>
       <c r="N19" s="38"/>
-    </row>
-    <row r="20" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P19" s="74"/>
+      <c r="Q19" s="68"/>
+      <c r="AT19"/>
+      <c r="AV19" s="68"/>
+    </row>
+    <row r="20" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M20" s="38"/>
       <c r="N20" s="38"/>
-    </row>
-    <row r="21" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P20" s="74"/>
+      <c r="Q20" s="68"/>
+      <c r="AT20"/>
+      <c r="AV20" s="68"/>
+    </row>
+    <row r="21" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M21" s="38"/>
       <c r="N21" s="38"/>
-    </row>
-    <row r="22" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P21" s="74"/>
+      <c r="Q21" s="68"/>
+      <c r="AT21"/>
+      <c r="AV21" s="68"/>
+    </row>
+    <row r="22" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M22" s="38"/>
       <c r="N22" s="38"/>
-    </row>
-    <row r="23" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P22" s="74"/>
+      <c r="Q22" s="68"/>
+      <c r="AT22"/>
+      <c r="AV22" s="68"/>
+    </row>
+    <row r="23" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M23" s="38"/>
       <c r="N23" s="38"/>
-    </row>
-    <row r="24" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P23" s="74"/>
+      <c r="Q23" s="68"/>
+      <c r="AT23"/>
+      <c r="AV23" s="68"/>
+    </row>
+    <row r="24" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M24" s="38"/>
       <c r="N24" s="38"/>
-    </row>
-    <row r="25" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P24" s="74"/>
+      <c r="Q24" s="68"/>
+      <c r="AT24"/>
+      <c r="AV24" s="68"/>
+    </row>
+    <row r="25" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M25" s="38"/>
       <c r="N25" s="38"/>
-    </row>
-    <row r="26" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P25" s="74"/>
+      <c r="Q25" s="68"/>
+      <c r="AT25"/>
+      <c r="AV25" s="68"/>
+    </row>
+    <row r="26" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M26" s="38"/>
       <c r="N26" s="38"/>
-    </row>
-    <row r="27" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P26" s="74"/>
+      <c r="Q26" s="68"/>
+      <c r="AT26"/>
+      <c r="AV26" s="68"/>
+    </row>
+    <row r="27" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M27" s="38"/>
       <c r="N27" s="38"/>
-    </row>
-    <row r="28" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P27" s="74"/>
+      <c r="Q27" s="68"/>
+      <c r="AT27"/>
+      <c r="AV27" s="68"/>
+    </row>
+    <row r="28" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M28" s="38"/>
       <c r="N28" s="38"/>
-    </row>
-    <row r="29" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P28" s="74"/>
+      <c r="Q28" s="68"/>
+      <c r="AT28"/>
+      <c r="AV28" s="68"/>
+    </row>
+    <row r="29" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M29" s="38"/>
       <c r="N29" s="38"/>
-    </row>
-    <row r="30" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P29" s="74"/>
+      <c r="Q29" s="68"/>
+      <c r="AT29"/>
+      <c r="AV29" s="68"/>
+    </row>
+    <row r="30" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M30" s="38"/>
       <c r="N30" s="38"/>
-    </row>
-    <row r="31" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P30" s="74"/>
+      <c r="Q30" s="68"/>
+      <c r="AT30"/>
+      <c r="AV30" s="68"/>
+    </row>
+    <row r="31" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M31" s="38"/>
       <c r="N31" s="38"/>
-    </row>
-    <row r="32" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P31" s="74"/>
+      <c r="Q31" s="68"/>
+      <c r="AT31"/>
+      <c r="AV31" s="68"/>
+    </row>
+    <row r="32" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M32" s="38"/>
       <c r="N32" s="38"/>
-    </row>
-    <row r="33" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P32" s="74"/>
+      <c r="Q32" s="68"/>
+      <c r="AT32"/>
+      <c r="AV32" s="68"/>
+    </row>
+    <row r="33" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M33" s="38"/>
       <c r="N33" s="38"/>
-    </row>
-    <row r="34" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P33" s="74"/>
+      <c r="Q33" s="68"/>
+      <c r="AT33"/>
+      <c r="AV33" s="68"/>
+    </row>
+    <row r="34" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M34" s="38"/>
       <c r="N34" s="38"/>
-    </row>
-    <row r="35" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P34" s="74"/>
+      <c r="Q34" s="68"/>
+      <c r="AT34"/>
+      <c r="AV34" s="68"/>
+    </row>
+    <row r="35" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M35" s="38"/>
       <c r="N35" s="38"/>
-    </row>
-    <row r="36" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P35" s="74"/>
+      <c r="Q35" s="68"/>
+      <c r="AT35"/>
+      <c r="AV35" s="68"/>
+    </row>
+    <row r="36" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M36" s="38"/>
       <c r="N36" s="38"/>
-    </row>
-    <row r="37" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P36" s="74"/>
+      <c r="Q36" s="68"/>
+      <c r="AT36"/>
+      <c r="AV36" s="68"/>
+    </row>
+    <row r="37" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M37" s="38"/>
       <c r="N37" s="38"/>
-    </row>
-    <row r="38" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P37" s="74"/>
+      <c r="Q37" s="68"/>
+      <c r="AT37"/>
+      <c r="AV37" s="68"/>
+    </row>
+    <row r="38" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M38" s="38"/>
       <c r="N38" s="38"/>
-    </row>
-    <row r="39" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P38" s="74"/>
+      <c r="Q38" s="68"/>
+      <c r="AT38"/>
+      <c r="AV38" s="68"/>
+    </row>
+    <row r="39" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M39" s="38"/>
       <c r="N39" s="38"/>
-    </row>
-    <row r="40" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P39" s="74"/>
+      <c r="Q39" s="68"/>
+      <c r="AT39"/>
+      <c r="AV39" s="68"/>
+    </row>
+    <row r="40" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M40" s="38"/>
       <c r="N40" s="38"/>
-    </row>
-    <row r="41" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P40" s="74"/>
+      <c r="Q40" s="68"/>
+      <c r="AT40"/>
+      <c r="AV40" s="68"/>
+    </row>
+    <row r="41" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M41" s="38"/>
       <c r="N41" s="38"/>
-    </row>
-    <row r="42" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P41" s="74"/>
+      <c r="Q41" s="68"/>
+      <c r="AT41"/>
+      <c r="AV41" s="68"/>
+    </row>
+    <row r="42" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M42" s="38"/>
       <c r="N42" s="38"/>
-    </row>
-    <row r="43" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P42" s="74"/>
+      <c r="Q42" s="68"/>
+      <c r="AT42"/>
+      <c r="AV42" s="68"/>
+    </row>
+    <row r="43" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M43" s="38"/>
       <c r="N43" s="38"/>
-    </row>
-    <row r="44" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P43" s="74"/>
+      <c r="Q43" s="68"/>
+      <c r="AT43"/>
+      <c r="AV43" s="68"/>
+    </row>
+    <row r="44" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M44" s="38"/>
       <c r="N44" s="38"/>
-    </row>
-    <row r="45" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P44" s="74"/>
+      <c r="Q44" s="68"/>
+      <c r="AT44"/>
+      <c r="AV44" s="68"/>
+    </row>
+    <row r="45" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M45" s="38"/>
       <c r="N45" s="38"/>
-    </row>
-    <row r="46" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P45" s="74"/>
+      <c r="Q45" s="68"/>
+      <c r="AT45"/>
+      <c r="AV45" s="68"/>
+    </row>
+    <row r="46" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M46" s="38"/>
       <c r="N46" s="38"/>
-    </row>
-    <row r="47" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P46" s="74"/>
+      <c r="Q46" s="68"/>
+      <c r="AT46"/>
+      <c r="AV46" s="68"/>
+    </row>
+    <row r="47" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M47" s="38"/>
       <c r="N47" s="38"/>
-    </row>
-    <row r="48" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P47" s="74"/>
+      <c r="Q47" s="68"/>
+      <c r="AT47"/>
+      <c r="AV47" s="68"/>
+    </row>
+    <row r="48" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M48" s="38"/>
       <c r="N48" s="38"/>
-    </row>
-    <row r="49" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P48" s="74"/>
+      <c r="Q48" s="68"/>
+      <c r="AT48"/>
+      <c r="AV48" s="68"/>
+    </row>
+    <row r="49" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M49" s="38"/>
       <c r="N49" s="38"/>
-    </row>
-    <row r="50" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P49" s="74"/>
+      <c r="Q49" s="68"/>
+      <c r="AT49"/>
+      <c r="AV49" s="68"/>
+    </row>
+    <row r="50" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M50" s="38"/>
       <c r="N50" s="38"/>
-    </row>
-    <row r="51" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P50" s="74"/>
+      <c r="Q50" s="68"/>
+      <c r="AT50"/>
+      <c r="AV50" s="68"/>
+    </row>
+    <row r="51" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M51" s="38"/>
       <c r="N51" s="38"/>
-    </row>
-    <row r="52" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P51" s="74"/>
+      <c r="Q51" s="68"/>
+      <c r="AT51"/>
+      <c r="AV51" s="68"/>
+    </row>
+    <row r="52" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M52" s="38"/>
       <c r="N52" s="38"/>
-    </row>
-    <row r="53" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P52" s="74"/>
+      <c r="Q52" s="68"/>
+      <c r="AT52"/>
+      <c r="AV52" s="68"/>
+    </row>
+    <row r="53" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M53" s="38"/>
       <c r="N53" s="38"/>
-    </row>
-    <row r="54" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P53" s="74"/>
+      <c r="Q53" s="68"/>
+      <c r="AT53"/>
+      <c r="AV53" s="68"/>
+    </row>
+    <row r="54" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M54" s="38"/>
       <c r="N54" s="38"/>
-    </row>
-    <row r="55" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P54" s="74"/>
+      <c r="Q54" s="68"/>
+      <c r="AT54"/>
+      <c r="AV54" s="68"/>
+    </row>
+    <row r="55" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M55" s="38"/>
       <c r="N55" s="38"/>
-    </row>
-    <row r="56" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P55" s="74"/>
+      <c r="Q55" s="68"/>
+      <c r="AT55"/>
+      <c r="AV55" s="68"/>
+    </row>
+    <row r="56" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M56" s="38"/>
       <c r="N56" s="38"/>
-    </row>
-    <row r="57" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P56" s="74"/>
+      <c r="Q56" s="68"/>
+      <c r="AT56"/>
+      <c r="AV56" s="68"/>
+    </row>
+    <row r="57" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M57" s="38"/>
       <c r="N57" s="38"/>
-    </row>
-    <row r="58" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P57" s="74"/>
+      <c r="Q57" s="68"/>
+      <c r="AT57"/>
+      <c r="AV57" s="68"/>
+    </row>
+    <row r="58" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M58" s="38"/>
       <c r="N58" s="38"/>
-    </row>
-    <row r="59" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P58" s="74"/>
+      <c r="Q58" s="68"/>
+      <c r="AT58"/>
+      <c r="AV58" s="68"/>
+    </row>
+    <row r="59" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M59" s="38"/>
       <c r="N59" s="38"/>
-    </row>
-    <row r="60" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P59" s="74"/>
+      <c r="Q59" s="68"/>
+      <c r="AT59"/>
+      <c r="AV59" s="68"/>
+    </row>
+    <row r="60" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M60" s="38"/>
       <c r="N60" s="38"/>
-    </row>
-    <row r="61" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P60" s="74"/>
+      <c r="Q60" s="68"/>
+      <c r="AT60"/>
+      <c r="AV60" s="68"/>
+    </row>
+    <row r="61" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M61" s="38"/>
       <c r="N61" s="38"/>
-    </row>
-    <row r="62" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P61" s="74"/>
+      <c r="Q61" s="68"/>
+      <c r="AT61"/>
+      <c r="AV61" s="68"/>
+    </row>
+    <row r="62" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M62" s="38"/>
       <c r="N62" s="38"/>
-    </row>
-    <row r="63" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P62" s="74"/>
+      <c r="Q62" s="68"/>
+      <c r="AT62"/>
+      <c r="AV62" s="68"/>
+    </row>
+    <row r="63" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M63" s="38"/>
       <c r="N63" s="38"/>
-    </row>
-    <row r="64" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P63" s="74"/>
+      <c r="Q63" s="68"/>
+      <c r="AT63"/>
+      <c r="AV63" s="68"/>
+    </row>
+    <row r="64" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M64" s="38"/>
       <c r="N64" s="38"/>
-    </row>
-    <row r="65" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P64" s="74"/>
+      <c r="Q64" s="68"/>
+      <c r="AT64"/>
+      <c r="AV64" s="68"/>
+    </row>
+    <row r="65" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M65" s="38"/>
       <c r="N65" s="38"/>
-    </row>
-    <row r="66" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P65" s="74"/>
+      <c r="Q65" s="68"/>
+      <c r="AT65"/>
+      <c r="AV65" s="68"/>
+    </row>
+    <row r="66" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M66" s="38"/>
       <c r="N66" s="38"/>
-    </row>
-    <row r="67" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P66" s="74"/>
+      <c r="Q66" s="68"/>
+      <c r="AT66"/>
+      <c r="AV66" s="68"/>
+    </row>
+    <row r="67" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M67" s="38"/>
       <c r="N67" s="38"/>
-    </row>
-    <row r="68" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P67" s="74"/>
+      <c r="Q67" s="68"/>
+      <c r="AT67"/>
+      <c r="AV67" s="68"/>
+    </row>
+    <row r="68" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M68" s="38"/>
       <c r="N68" s="38"/>
-    </row>
-    <row r="69" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P68" s="74"/>
+      <c r="Q68" s="68"/>
+      <c r="AT68"/>
+      <c r="AV68" s="68"/>
+    </row>
+    <row r="69" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M69" s="38"/>
       <c r="N69" s="38"/>
-    </row>
-    <row r="70" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P69" s="74"/>
+      <c r="Q69" s="68"/>
+      <c r="AT69"/>
+      <c r="AV69" s="68"/>
+    </row>
+    <row r="70" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M70" s="38"/>
       <c r="N70" s="38"/>
-    </row>
-    <row r="71" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P70" s="74"/>
+      <c r="Q70" s="68"/>
+      <c r="AT70"/>
+      <c r="AV70" s="68"/>
+    </row>
+    <row r="71" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M71" s="38"/>
       <c r="N71" s="38"/>
-    </row>
-    <row r="72" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P71" s="74"/>
+      <c r="Q71" s="68"/>
+      <c r="AT71"/>
+      <c r="AV71" s="68"/>
+    </row>
+    <row r="72" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M72" s="38"/>
       <c r="N72" s="38"/>
-    </row>
-    <row r="73" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P72" s="74"/>
+      <c r="Q72" s="68"/>
+      <c r="AT72"/>
+      <c r="AV72" s="68"/>
+    </row>
+    <row r="73" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M73" s="38"/>
       <c r="N73" s="38"/>
-    </row>
-    <row r="74" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P73" s="74"/>
+      <c r="Q73" s="68"/>
+      <c r="AT73"/>
+      <c r="AV73" s="68"/>
+    </row>
+    <row r="74" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M74" s="38"/>
       <c r="N74" s="38"/>
-    </row>
-    <row r="75" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P74" s="74"/>
+      <c r="Q74" s="68"/>
+      <c r="AT74"/>
+      <c r="AV74" s="68"/>
+    </row>
+    <row r="75" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M75" s="38"/>
       <c r="N75" s="38"/>
-    </row>
-    <row r="76" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P75" s="74"/>
+      <c r="Q75" s="68"/>
+      <c r="AT75"/>
+      <c r="AV75" s="68"/>
+    </row>
+    <row r="76" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M76" s="38"/>
       <c r="N76" s="38"/>
-    </row>
-    <row r="77" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P76" s="74"/>
+      <c r="Q76" s="68"/>
+      <c r="AT76"/>
+      <c r="AV76" s="68"/>
+    </row>
+    <row r="77" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M77" s="38"/>
       <c r="N77" s="38"/>
-    </row>
-    <row r="78" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P77" s="74"/>
+      <c r="Q77" s="68"/>
+      <c r="AT77"/>
+      <c r="AV77" s="68"/>
+    </row>
+    <row r="78" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M78" s="38"/>
       <c r="N78" s="38"/>
-    </row>
-    <row r="79" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P78" s="74"/>
+      <c r="Q78" s="68"/>
+      <c r="AT78"/>
+      <c r="AV78" s="68"/>
+    </row>
+    <row r="79" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M79" s="38"/>
       <c r="N79" s="38"/>
-    </row>
-    <row r="80" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P79" s="74"/>
+      <c r="Q79" s="68"/>
+      <c r="AT79"/>
+      <c r="AV79" s="68"/>
+    </row>
+    <row r="80" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M80" s="38"/>
       <c r="N80" s="38"/>
-    </row>
-    <row r="81" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P80" s="74"/>
+      <c r="Q80" s="68"/>
+      <c r="AT80"/>
+      <c r="AV80" s="68"/>
+    </row>
+    <row r="81" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M81" s="38"/>
       <c r="N81" s="38"/>
-    </row>
-    <row r="82" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P81" s="74"/>
+      <c r="Q81" s="68"/>
+      <c r="AT81"/>
+      <c r="AV81" s="68"/>
+    </row>
+    <row r="82" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M82" s="38"/>
       <c r="N82" s="38"/>
-    </row>
-    <row r="83" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P82" s="74"/>
+      <c r="Q82" s="68"/>
+      <c r="AT82"/>
+      <c r="AV82" s="68"/>
+    </row>
+    <row r="83" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M83" s="38"/>
       <c r="N83" s="38"/>
-    </row>
-    <row r="84" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P83" s="74"/>
+      <c r="Q83" s="68"/>
+      <c r="AT83"/>
+      <c r="AV83" s="68"/>
+    </row>
+    <row r="84" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M84" s="38"/>
       <c r="N84" s="38"/>
-    </row>
-    <row r="85" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P84" s="74"/>
+      <c r="Q84" s="68"/>
+      <c r="AT84"/>
+      <c r="AV84" s="68"/>
+    </row>
+    <row r="85" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M85" s="38"/>
       <c r="N85" s="38"/>
-    </row>
-    <row r="86" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P85" s="74"/>
+      <c r="Q85" s="68"/>
+      <c r="AT85"/>
+      <c r="AV85" s="68"/>
+    </row>
+    <row r="86" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M86" s="38"/>
       <c r="N86" s="38"/>
-    </row>
-    <row r="87" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P86" s="74"/>
+      <c r="Q86" s="68"/>
+      <c r="AT86"/>
+      <c r="AV86" s="68"/>
+    </row>
+    <row r="87" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M87" s="38"/>
       <c r="N87" s="38"/>
-    </row>
-    <row r="88" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P87" s="74"/>
+      <c r="Q87" s="68"/>
+      <c r="AT87"/>
+      <c r="AV87" s="68"/>
+    </row>
+    <row r="88" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M88" s="38"/>
       <c r="N88" s="38"/>
-    </row>
-    <row r="89" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P88" s="74"/>
+      <c r="Q88" s="68"/>
+      <c r="AT88"/>
+      <c r="AV88" s="68"/>
+    </row>
+    <row r="89" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M89" s="38"/>
       <c r="N89" s="38"/>
-    </row>
-    <row r="90" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P89" s="74"/>
+      <c r="Q89" s="68"/>
+      <c r="AT89"/>
+      <c r="AV89" s="68"/>
+    </row>
+    <row r="90" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M90" s="38"/>
       <c r="N90" s="38"/>
-    </row>
-    <row r="91" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P90" s="74"/>
+      <c r="Q90" s="68"/>
+      <c r="AT90"/>
+      <c r="AV90" s="68"/>
+    </row>
+    <row r="91" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M91" s="38"/>
       <c r="N91" s="38"/>
-    </row>
-    <row r="92" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P91" s="74"/>
+      <c r="Q91" s="68"/>
+      <c r="AT91"/>
+      <c r="AV91" s="68"/>
+    </row>
+    <row r="92" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M92" s="38"/>
       <c r="N92" s="38"/>
-    </row>
-    <row r="93" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P92" s="74"/>
+      <c r="Q92" s="68"/>
+      <c r="AT92"/>
+      <c r="AV92" s="68"/>
+    </row>
+    <row r="93" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M93" s="38"/>
       <c r="N93" s="38"/>
-    </row>
-    <row r="94" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P93" s="74"/>
+      <c r="Q93" s="68"/>
+      <c r="AT93"/>
+      <c r="AV93" s="68"/>
+    </row>
+    <row r="94" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M94" s="38"/>
       <c r="N94" s="38"/>
-    </row>
-    <row r="95" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P94" s="74"/>
+      <c r="Q94" s="68"/>
+      <c r="AT94"/>
+      <c r="AV94" s="68"/>
+    </row>
+    <row r="95" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M95" s="38"/>
       <c r="N95" s="38"/>
-    </row>
-    <row r="96" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P95" s="74"/>
+      <c r="Q95" s="68"/>
+      <c r="AT95"/>
+      <c r="AV95" s="68"/>
+    </row>
+    <row r="96" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M96" s="38"/>
       <c r="N96" s="38"/>
-    </row>
-    <row r="97" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P96" s="74"/>
+      <c r="Q96" s="68"/>
+      <c r="AT96"/>
+      <c r="AV96" s="68"/>
+    </row>
+    <row r="97" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M97" s="38"/>
       <c r="N97" s="38"/>
-    </row>
-    <row r="98" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P97" s="74"/>
+      <c r="Q97" s="68"/>
+      <c r="AT97"/>
+      <c r="AV97" s="68"/>
+    </row>
+    <row r="98" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M98" s="38"/>
       <c r="N98" s="38"/>
-    </row>
-    <row r="99" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P98" s="74"/>
+      <c r="Q98" s="68"/>
+      <c r="AT98"/>
+      <c r="AV98" s="68"/>
+    </row>
+    <row r="99" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M99" s="38"/>
       <c r="N99" s="38"/>
-    </row>
-    <row r="100" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P99" s="74"/>
+      <c r="Q99" s="68"/>
+      <c r="AT99"/>
+      <c r="AV99" s="68"/>
+    </row>
+    <row r="100" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M100" s="38"/>
       <c r="N100" s="38"/>
+      <c r="P100" s="74"/>
+      <c r="Q100" s="68"/>
+      <c r="AT100"/>
+      <c r="AV100" s="68"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="H1:J1"/>
-    <mergeCell ref="P1:AT1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2744,7 +3203,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="fertilizer" prompt="select type" xr:uid="{B70B515A-9E4D-43A4-A403-3B52F4B6E7A5}">
           <x14:formula1>
             <xm:f>options!$C$2:$C$9</xm:f>
@@ -2756,6 +3215,12 @@
             <xm:f>options!$E$2:$E$3</xm:f>
           </x14:formula1>
           <xm:sqref>N3:N100</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="irrigation location" prompt="Indicate if irrigation applied aboveground (either above or below plant canopy) or belowground (i.e. drip). " xr:uid="{D1AF471D-DDE0-4230-AA87-8B03F8E0C30A}">
+          <x14:formula1>
+            <xm:f>options!$K$2:$K$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>P3:P100</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2797,85 +3262,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:71" x14ac:dyDescent="0.3">
-      <c r="B1" s="56" t="s">
+      <c r="B1" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="52" t="s">
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="T1" s="52"/>
-      <c r="U1" s="52"/>
-      <c r="V1" s="52"/>
-      <c r="W1" s="52"/>
-      <c r="X1" s="52"/>
-      <c r="Y1" s="52"/>
-      <c r="Z1" s="52"/>
-      <c r="AA1" s="52"/>
-      <c r="AB1" s="52"/>
-      <c r="AC1" s="52"/>
-      <c r="AD1" s="52"/>
-      <c r="AE1" s="52"/>
-      <c r="AF1" s="51" t="s">
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
+      <c r="W1" s="56"/>
+      <c r="X1" s="56"/>
+      <c r="Y1" s="56"/>
+      <c r="Z1" s="56"/>
+      <c r="AA1" s="56"/>
+      <c r="AB1" s="56"/>
+      <c r="AC1" s="56"/>
+      <c r="AD1" s="56"/>
+      <c r="AE1" s="56"/>
+      <c r="AF1" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="AG1" s="51"/>
-      <c r="AH1" s="51"/>
-      <c r="AI1" s="51"/>
-      <c r="AJ1" s="51"/>
-      <c r="AK1" s="51"/>
-      <c r="AL1" s="51"/>
-      <c r="AM1" s="51"/>
-      <c r="AN1" s="51"/>
-      <c r="AO1" s="51"/>
-      <c r="AP1" s="51"/>
-      <c r="AQ1" s="51"/>
-      <c r="AR1" s="51"/>
-      <c r="AS1" s="55" t="s">
+      <c r="AG1" s="55"/>
+      <c r="AH1" s="55"/>
+      <c r="AI1" s="55"/>
+      <c r="AJ1" s="55"/>
+      <c r="AK1" s="55"/>
+      <c r="AL1" s="55"/>
+      <c r="AM1" s="55"/>
+      <c r="AN1" s="55"/>
+      <c r="AO1" s="55"/>
+      <c r="AP1" s="55"/>
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="55"/>
+      <c r="AS1" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="AT1" s="55"/>
-      <c r="AU1" s="55"/>
-      <c r="AV1" s="55"/>
-      <c r="AW1" s="55"/>
-      <c r="AX1" s="55"/>
-      <c r="AY1" s="55"/>
-      <c r="AZ1" s="55"/>
-      <c r="BA1" s="55"/>
-      <c r="BB1" s="55"/>
-      <c r="BC1" s="55"/>
-      <c r="BD1" s="55"/>
-      <c r="BE1" s="57"/>
-      <c r="BF1" s="58" t="s">
-        <v>150</v>
-      </c>
-      <c r="BG1" s="58"/>
-      <c r="BH1" s="58"/>
-      <c r="BI1" s="58"/>
-      <c r="BJ1" s="58"/>
-      <c r="BK1" s="58"/>
-      <c r="BL1" s="58"/>
-      <c r="BM1" s="58"/>
-      <c r="BN1" s="58"/>
-      <c r="BO1" s="58"/>
-      <c r="BP1" s="58"/>
-      <c r="BQ1" s="58"/>
-      <c r="BR1" s="59"/>
+      <c r="AT1" s="59"/>
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="59"/>
+      <c r="AW1" s="59"/>
+      <c r="AX1" s="59"/>
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="59"/>
+      <c r="BA1" s="59"/>
+      <c r="BB1" s="59"/>
+      <c r="BC1" s="59"/>
+      <c r="BD1" s="59"/>
+      <c r="BE1" s="61"/>
+      <c r="BF1" s="62" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG1" s="62"/>
+      <c r="BH1" s="62"/>
+      <c r="BI1" s="62"/>
+      <c r="BJ1" s="62"/>
+      <c r="BK1" s="62"/>
+      <c r="BL1" s="62"/>
+      <c r="BM1" s="62"/>
+      <c r="BN1" s="62"/>
+      <c r="BO1" s="62"/>
+      <c r="BP1" s="62"/>
+      <c r="BQ1" s="62"/>
+      <c r="BR1" s="63"/>
     </row>
     <row r="2" spans="1:71" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
@@ -2888,7 +3353,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>11</v>
@@ -2900,40 +3365,40 @@
         <v>13</v>
       </c>
       <c r="H2" s="27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I2" s="27" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="K2" s="27" t="s">
         <v>126</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>127</v>
       </c>
       <c r="L2" s="27" t="s">
         <v>43</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N2" s="27" t="s">
         <v>44</v>
       </c>
       <c r="O2" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P2" s="27" t="s">
         <v>15</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R2" s="29" t="s">
         <v>16</v>
       </c>
       <c r="S2" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="T2" s="30" t="s">
         <v>18</v>
@@ -2954,25 +3419,25 @@
         <v>45</v>
       </c>
       <c r="Z2" s="24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>46</v>
       </c>
       <c r="AB2" s="24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC2" s="30" t="s">
         <v>23</v>
       </c>
       <c r="AD2" s="24" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AE2" s="31" t="s">
         <v>24</v>
       </c>
       <c r="AF2" s="25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG2" s="32" t="s">
         <v>25</v>
@@ -2993,25 +3458,25 @@
         <v>47</v>
       </c>
       <c r="AM2" s="34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AN2" s="32" t="s">
         <v>48</v>
       </c>
       <c r="AO2" s="34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AP2" s="32" t="s">
         <v>30</v>
       </c>
       <c r="AQ2" s="34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AR2" s="33" t="s">
         <v>31</v>
       </c>
       <c r="AS2" s="35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AT2" s="36" t="s">
         <v>32</v>
@@ -3032,64 +3497,64 @@
         <v>49</v>
       </c>
       <c r="AZ2" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="BA2" s="36" t="s">
         <v>50</v>
       </c>
       <c r="BB2" s="37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="BC2" s="36" t="s">
         <v>37</v>
       </c>
       <c r="BD2" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BE2" s="36" t="s">
         <v>38</v>
       </c>
       <c r="BF2" s="44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="BG2" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="BH2" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="BH2" s="46" t="s">
+      <c r="BI2" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="BI2" s="46" t="s">
+      <c r="BJ2" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="BJ2" s="46" t="s">
+      <c r="BK2" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="BK2" s="46" t="s">
+      <c r="BL2" s="46" t="s">
         <v>155</v>
       </c>
-      <c r="BL2" s="46" t="s">
+      <c r="BM2" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="BM2" s="47" t="s">
+      <c r="BN2" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="BN2" s="46" t="s">
+      <c r="BO2" s="47" t="s">
         <v>158</v>
       </c>
-      <c r="BO2" s="47" t="s">
+      <c r="BP2" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="BP2" s="46" t="s">
+      <c r="BQ2" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="BQ2" s="47" t="s">
+      <c r="BR2" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="BR2" s="46" t="s">
+      <c r="BS2" s="48" t="s">
         <v>162</v>
-      </c>
-      <c r="BS2" s="48" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:71" x14ac:dyDescent="0.3">
@@ -6477,16 +6942,16 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C1"/>
-      <c r="D1" s="60" t="s">
+      <c r="D1" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="61"/>
-      <c r="I1" s="62" t="s">
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="67"/>
+      <c r="I1" s="64" t="s">
         <v>86</v>
       </c>
-      <c r="J1" s="63"/>
+      <c r="J1" s="65"/>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
@@ -7061,23 +7526,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>91</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D1" s="53" t="s">
         <v>164</v>
       </c>
-      <c r="D1" s="66" t="s">
+      <c r="E1" s="51" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="51" t="s">
         <v>165</v>
-      </c>
-      <c r="E1" s="64" t="s">
-        <v>167</v>
-      </c>
-      <c r="F1" s="64" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -7189,7 +7654,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA73EF4-F459-4FB8-999B-97CF29F368C2}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" customWidth="1"/>
@@ -7197,9 +7662,10 @@
     <col min="5" max="5" width="20.44140625" customWidth="1"/>
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="11" max="11" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>72</v>
       </c>
@@ -7210,13 +7676,16 @@
         <v>74</v>
       </c>
       <c r="G1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="K1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -7227,13 +7696,16 @@
         <v>75</v>
       </c>
       <c r="G2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+      <c r="K2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -7244,21 +7716,27 @@
         <v>76</v>
       </c>
       <c r="G3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+      <c r="K3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>70</v>
       </c>
       <c r="C4" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -7266,37 +7744,38 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="5">
+  <tableParts count="6">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added functions convert_dates, is_excel_date, get_code_choice. Updated date_to_jul. Moved conversion funtions to convert.R. Added globals.R
</commit_message>
<xml_diff>
--- a/files/Templates/collected_data.xlsx
+++ b/files/Templates/collected_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpo\Documents\Research\STICS\Code\mkSTICSfiles\files\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpo\Documents\Research\STICS\Code\mkSTICSfiles\files\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8435BD-6E33-4294-89A4-E4A9A779B45D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424D330F-59F3-4D69-84F8-7B0E19D330F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="30936" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="management" sheetId="8" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="stations" sheetId="6" r:id="rId3"/>
     <sheet name="usms" sheetId="1" r:id="rId4"/>
     <sheet name="observations" sheetId="9" r:id="rId5"/>
-    <sheet name="options" sheetId="4" state="hidden" r:id="rId6"/>
+    <sheet name="options" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Fertilizer_Application">Table3[Fertilizer_Application]</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="178">
   <si>
     <t>usm_name</t>
   </si>
@@ -421,9 +421,6 @@
     <t>amount_15</t>
   </si>
   <si>
-    <t>irrigation_date_16</t>
-  </si>
-  <si>
     <t>Irrigation</t>
   </si>
   <si>
@@ -557,6 +554,36 @@
   </si>
   <si>
     <t>albedo</t>
+  </si>
+  <si>
+    <t>harvest_end</t>
+  </si>
+  <si>
+    <t>harvest_date2</t>
+  </si>
+  <si>
+    <t>automatic_irr_depth</t>
+  </si>
+  <si>
+    <t>harvest</t>
+  </si>
+  <si>
+    <t>irrigation_type</t>
+  </si>
+  <si>
+    <t>irr_efficiency</t>
+  </si>
+  <si>
+    <t>Irrigation Location</t>
+  </si>
+  <si>
+    <t>1 = above the foliage</t>
+  </si>
+  <si>
+    <t>2 = below the foliage above the soil</t>
+  </si>
+  <si>
+    <t>3 = in the soil</t>
   </si>
 </sst>
 </file>
@@ -601,7 +628,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,6 +785,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="gray0625">
+        <fgColor theme="0" tint="-0.14993743705557422"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="14">
     <border>
@@ -908,7 +941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -962,6 +995,10 @@
     <xf numFmtId="0" fontId="3" fillId="26" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -989,122 +1026,30 @@
     <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="55">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -1166,76 +1111,6 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray0625">
-          <fgColor theme="0" tint="-0.24994659260841701"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1565,6 +1440,171 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray0625">
+          <fgColor theme="0" tint="-0.24994659260841701"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1591,24 +1631,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}" name="Table6" displayName="Table6" ref="A2:AT100" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7">
-  <autoFilter ref="A2:AT100" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}"/>
-  <tableColumns count="46">
-    <tableColumn id="1" xr3:uid="{6B129591-A0EC-4CC8-AA8E-70259B5C9131}" name="file_name" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{1FBFF361-0229-404E-A60E-FCEC995B36AD}" name="year" dataDxfId="4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}" name="Table6" displayName="Table6" ref="A2:AX100" totalsRowShown="0" headerRowDxfId="48" headerRowBorderDxfId="47" tableBorderDxfId="46">
+  <autoFilter ref="A2:AX100" xr:uid="{1AD7F1BC-9C4F-46C6-88D5-D2D5C340F1D9}"/>
+  <tableColumns count="50">
+    <tableColumn id="1" xr3:uid="{6B129591-A0EC-4CC8-AA8E-70259B5C9131}" name="file_name" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{1FBFF361-0229-404E-A60E-FCEC995B36AD}" name="year" dataDxfId="44"/>
     <tableColumn id="3" xr3:uid="{416116E5-319A-4096-B7E5-AF8ADEF0E80A}" name="tillage_date"/>
-    <tableColumn id="4" xr3:uid="{781FB9F7-258C-4E50-8A90-CAA110FA989E}" name="tillage_depth" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{781FB9F7-258C-4E50-8A90-CAA110FA989E}" name="tillage_depth" dataDxfId="43"/>
     <tableColumn id="5" xr3:uid="{A768ED69-1CCB-4A41-99C1-D5042177408B}" name="planting_date"/>
     <tableColumn id="6" xr3:uid="{5517C570-4D1C-46EC-9FB0-4FEA929440E1}" name="planting_depth"/>
-    <tableColumn id="7" xr3:uid="{8F3D9EFB-6197-44D6-9CAB-532096E5D0DE}" name="plants_per_m2" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{8F3D9EFB-6197-44D6-9CAB-532096E5D0DE}" name="plants_per_m2" dataDxfId="42"/>
     <tableColumn id="8" xr3:uid="{7DEB259C-DAE3-4A1E-B476-951FEF30ABD2}" name="emergence"/>
     <tableColumn id="9" xr3:uid="{8590CC43-CF1F-45A9-A612-CE3749B53C84}" name="flowering"/>
-    <tableColumn id="10" xr3:uid="{DAF1F67C-7CB4-4AD2-B1D4-24884C7C9D57}" name="maturity" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{DAF1F67C-7CB4-4AD2-B1D4-24884C7C9D57}" name="maturity" dataDxfId="41"/>
     <tableColumn id="11" xr3:uid="{1651DE3B-149A-4121-AFB0-BA33E8308050}" name="application_date"/>
     <tableColumn id="12" xr3:uid="{358B23A5-F859-4B79-9182-F98F3D69F461}" name="kg_N_per_ha"/>
     <tableColumn id="13" xr3:uid="{FEB67719-45D9-4389-A438-548C552EBED6}" name="fert_type"/>
     <tableColumn id="14" xr3:uid="{B9B3005C-6E63-4AA3-BE8E-646D9659B76F}" name="fert_location"/>
-    <tableColumn id="15" xr3:uid="{F5737449-F543-4637-B8F3-6DBD1B98EDA2}" name="fert_depth" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{F5737449-F543-4637-B8F3-6DBD1B98EDA2}" name="fert_depth" dataDxfId="40"/>
+    <tableColumn id="49" xr3:uid="{1DACF6E4-1D01-4D98-B61F-06AED8D28283}" name="irrigation_type"/>
+    <tableColumn id="48" xr3:uid="{E053F1CC-2741-44D0-BCB6-E2638B921A91}" name="irr_efficiency"/>
     <tableColumn id="16" xr3:uid="{AA12C7D8-D645-4337-B05C-CB5F5C197AE4}" name="irrigation_date_1"/>
     <tableColumn id="17" xr3:uid="{017BC113-D478-4E04-AEE6-020CA6B48738}" name="amount_1"/>
     <tableColumn id="18" xr3:uid="{498ED556-89DC-49A5-A6C1-DF741DBED2EF}" name="irrigation_date_2"/>
@@ -1639,7 +1681,9 @@
     <tableColumn id="43" xr3:uid="{0A0B6CAB-9EC9-4492-A667-1846AE54A020}" name="amount_14"/>
     <tableColumn id="44" xr3:uid="{7DD1FA19-1C12-4443-9EB3-267851A488BA}" name="irrigation_date_15"/>
     <tableColumn id="45" xr3:uid="{A69E1720-4BA7-4736-9E85-A0E33013B090}" name="amount_15"/>
-    <tableColumn id="46" xr3:uid="{A0DFD622-ADA5-48E2-B689-A17242FFBEEA}" name="irrigation_date_16"/>
+    <tableColumn id="51" xr3:uid="{D644A008-911D-42DE-B5AE-3D97E8D9CBE3}" name="automatic_irr_depth"/>
+    <tableColumn id="47" xr3:uid="{8142D301-45D6-476E-91F5-4C775D8382CE}" name="harvest_date2"/>
+    <tableColumn id="50" xr3:uid="{A3119A2B-1FF4-4688-A8C7-EA84F5130A56}" name="harvest_end"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1655,11 +1699,21 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{EC7F3CD2-B7DD-4AB9-A1D1-61C6B8E31CF2}" name="Table11" displayName="Table11" ref="K1:K4" totalsRowShown="0">
+  <autoFilter ref="K1:K4" xr:uid="{EC7F3CD2-B7DD-4AB9-A1D1-61C6B8E31CF2}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{684BC5C4-FC4C-4A03-9843-BEAD87C7E594}" name="Irrigation Location"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}" name="Table7" displayName="Table7" ref="A2:BS100" totalsRowShown="0" headerRowDxfId="54" headerRowBorderDxfId="53" tableBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}" name="Table7" displayName="Table7" ref="A2:BS100" totalsRowShown="0" headerRowDxfId="39" headerRowBorderDxfId="38" tableBorderDxfId="37">
   <autoFilter ref="A2:BS100" xr:uid="{34F446AA-1543-42D0-AA83-3EA91742E62F}"/>
   <tableColumns count="71">
-    <tableColumn id="1" xr3:uid="{4674EE1C-2CD4-485E-8B27-A14DEFFAAD8A}" name="soil_profile_name" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{4674EE1C-2CD4-485E-8B27-A14DEFFAAD8A}" name="soil_profile_name" dataDxfId="36"/>
     <tableColumn id="2" xr3:uid="{72D785FE-A1AF-4E08-AB14-39FAD15DB9BD}" name="thickness_1"/>
     <tableColumn id="3" xr3:uid="{1838D7E8-2B3C-471C-9A0B-D70D91F18417}" name="pH"/>
     <tableColumn id="71" xr3:uid="{931F79EB-F524-439C-8A88-ED674075FA7F}" name="albedo"/>
@@ -1671,110 +1725,110 @@
     <tableColumn id="40" xr3:uid="{EC836542-6DD7-49C9-82D9-B724BCE18341}" name="SON_1"/>
     <tableColumn id="41" xr3:uid="{F7750E58-5B0E-4494-87AF-B025671824DE}" name="CN_ratio"/>
     <tableColumn id="8" xr3:uid="{0592115C-328E-42C4-B9CB-D43026D4FC27}" name="FC_1"/>
-    <tableColumn id="42" xr3:uid="{5C21A417-1737-43F1-BC15-EC087A009A68}" name="FC_1_unit" dataDxfId="50"/>
+    <tableColumn id="42" xr3:uid="{5C21A417-1737-43F1-BC15-EC087A009A68}" name="FC_1_unit" dataDxfId="35"/>
     <tableColumn id="9" xr3:uid="{C1383A59-387E-4667-852A-B0CF467088F3}" name="WP_1"/>
-    <tableColumn id="43" xr3:uid="{75E60C07-9873-41B6-AB5A-253087B95CFA}" name="WP_1_unit" dataDxfId="49"/>
+    <tableColumn id="43" xr3:uid="{75E60C07-9873-41B6-AB5A-253087B95CFA}" name="WP_1_unit" dataDxfId="34"/>
     <tableColumn id="10" xr3:uid="{34D0D911-5DB4-457F-88A7-76A42B57EE1A}" name="initial_NO3_1"/>
-    <tableColumn id="52" xr3:uid="{630D852C-736F-4D0D-8BB3-6EB32B59A383}" name="initial_NO3_1_units" dataDxfId="48"/>
+    <tableColumn id="52" xr3:uid="{630D852C-736F-4D0D-8BB3-6EB32B59A383}" name="initial_NO3_1_units" dataDxfId="33"/>
     <tableColumn id="53" xr3:uid="{CEF78893-60AA-4A20-A771-E76562B8EBC1}" name="initial_NH4_1"/>
-    <tableColumn id="11" xr3:uid="{58B6280A-10C4-4120-9FF8-93150CE70C6B}" name="initial_NH4_1_units" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{58B6280A-10C4-4120-9FF8-93150CE70C6B}" name="initial_NH4_1_units" dataDxfId="32"/>
     <tableColumn id="12" xr3:uid="{FD043EB5-2678-4920-8D76-EBE8316E27AA}" name="thickness_2"/>
     <tableColumn id="13" xr3:uid="{F124AE04-B447-4F21-A0E8-7B26199C0F49}" name="%_sand_2"/>
     <tableColumn id="14" xr3:uid="{F119498A-3A35-40E3-A753-7CF13D724118}" name="%_clay_2"/>
     <tableColumn id="15" xr3:uid="{AE51522F-6903-42D4-88CE-A95BCE8C77EF}" name="BD_2"/>
     <tableColumn id="16" xr3:uid="{12076489-6AD7-4297-A729-20EF93AEE58D}" name="SOC_2"/>
     <tableColumn id="17" xr3:uid="{D6D5EFD4-69CC-4AF2-8C6B-0B430468C4C2}" name="FC_2"/>
-    <tableColumn id="44" xr3:uid="{7158FD96-C69C-40D1-A3B8-2D043DF66D42}" name="FC_2_unit" dataDxfId="46"/>
+    <tableColumn id="44" xr3:uid="{7158FD96-C69C-40D1-A3B8-2D043DF66D42}" name="FC_2_unit" dataDxfId="31"/>
     <tableColumn id="18" xr3:uid="{BBF6A61D-2092-4DF7-8C38-9024164291AE}" name="WP_2"/>
-    <tableColumn id="45" xr3:uid="{2A662E87-2699-41FA-AF9F-C807E1C2112B}" name="WP_2_unit" dataDxfId="45"/>
+    <tableColumn id="45" xr3:uid="{2A662E87-2699-41FA-AF9F-C807E1C2112B}" name="WP_2_unit" dataDxfId="30"/>
     <tableColumn id="19" xr3:uid="{BB4B796C-CA3E-424C-87B0-4BF33581B61B}" name="initial_NO3_2"/>
-    <tableColumn id="54" xr3:uid="{13CDB225-A28A-424D-943F-330A6ABE0CF2}" name="initial_NO3_2_unit" dataDxfId="44"/>
+    <tableColumn id="54" xr3:uid="{13CDB225-A28A-424D-943F-330A6ABE0CF2}" name="initial_NO3_2_unit" dataDxfId="29"/>
     <tableColumn id="55" xr3:uid="{333E59C3-3A13-4C92-9169-AC90D5E5D3EB}" name="initial_NH4_2"/>
-    <tableColumn id="20" xr3:uid="{613F6ECB-AFEC-4E8A-BD78-2579E90B1783}" name="initial_NH4_2_unit" dataDxfId="43"/>
-    <tableColumn id="21" xr3:uid="{5D7B3549-7F90-410E-90FF-149F4376EBB7}" name="thickness_3" dataDxfId="42"/>
+    <tableColumn id="20" xr3:uid="{613F6ECB-AFEC-4E8A-BD78-2579E90B1783}" name="initial_NH4_2_unit" dataDxfId="28"/>
+    <tableColumn id="21" xr3:uid="{5D7B3549-7F90-410E-90FF-149F4376EBB7}" name="thickness_3" dataDxfId="27"/>
     <tableColumn id="22" xr3:uid="{6C917DE4-8D95-496E-A6F1-EAB7450774EE}" name="%_sand_3"/>
     <tableColumn id="23" xr3:uid="{90DE7FE2-3A23-4294-8BD0-2D321FF71179}" name="%_clay_3"/>
     <tableColumn id="24" xr3:uid="{C874CBBB-CB06-4239-AE9B-72564A3EDC14}" name="BD_3"/>
     <tableColumn id="25" xr3:uid="{49CED3FB-E83C-4973-A99D-DAC6B3AFC7B1}" name="SOC_3"/>
     <tableColumn id="26" xr3:uid="{63FB3901-EBED-4379-9E9C-83064A8ADD01}" name="FC_3"/>
-    <tableColumn id="47" xr3:uid="{5C201AAC-779E-4362-9603-51762D2AD5CF}" name="FC_3_unit" dataDxfId="41"/>
+    <tableColumn id="47" xr3:uid="{5C201AAC-779E-4362-9603-51762D2AD5CF}" name="FC_3_unit" dataDxfId="26"/>
     <tableColumn id="27" xr3:uid="{6EEACF0E-3934-49DF-9991-42C2DB718BE0}" name="WP_3"/>
-    <tableColumn id="48" xr3:uid="{67EEF171-24DC-4B50-B1F4-746B04E8F368}" name="WP_3_unit" dataDxfId="40"/>
+    <tableColumn id="48" xr3:uid="{67EEF171-24DC-4B50-B1F4-746B04E8F368}" name="WP_3_unit" dataDxfId="25"/>
     <tableColumn id="28" xr3:uid="{7AAE3F1E-C60E-4E11-A023-F09548D5AA39}" name="initial_NO3_3"/>
-    <tableColumn id="56" xr3:uid="{2B23B0A6-3617-432B-8EEA-E2AC0892F317}" name="initial_NO3_3_unit" dataDxfId="39"/>
+    <tableColumn id="56" xr3:uid="{2B23B0A6-3617-432B-8EEA-E2AC0892F317}" name="initial_NO3_3_unit" dataDxfId="24"/>
     <tableColumn id="57" xr3:uid="{1D0A3587-38DB-4073-B5D4-36DA82425955}" name="initial_NH4_3"/>
-    <tableColumn id="29" xr3:uid="{4BF74EC8-B9F2-42F0-AA7F-7CF70391A1FD}" name="initial_NH4_3_unit" dataDxfId="38"/>
-    <tableColumn id="30" xr3:uid="{4F55D6E9-95FD-4FC3-8012-EBB0DDAD9C3D}" name="thickness_4" dataDxfId="37"/>
+    <tableColumn id="29" xr3:uid="{4BF74EC8-B9F2-42F0-AA7F-7CF70391A1FD}" name="initial_NH4_3_unit" dataDxfId="23"/>
+    <tableColumn id="30" xr3:uid="{4F55D6E9-95FD-4FC3-8012-EBB0DDAD9C3D}" name="thickness_4" dataDxfId="22"/>
     <tableColumn id="31" xr3:uid="{4C1178FA-055B-4F19-A181-638D37A24EB6}" name="%_sand_4"/>
     <tableColumn id="32" xr3:uid="{7BBFA3FD-BBE5-4B68-A551-EFDEA7062540}" name="%_clay_4"/>
     <tableColumn id="33" xr3:uid="{D0607A27-FB9E-4DA9-A7F3-7A932B2608A4}" name="BD_4"/>
     <tableColumn id="34" xr3:uid="{BD46131F-AB56-411A-8742-B77FBBE1967B}" name="SOC_4"/>
     <tableColumn id="35" xr3:uid="{EC2EEDB8-3CC6-4DEE-9309-DBA3B11A2D16}" name="FC_4"/>
-    <tableColumn id="50" xr3:uid="{D1D16E63-48A7-4CF1-950A-55FD748CC035}" name="FC_4_unit" dataDxfId="36"/>
-    <tableColumn id="36" xr3:uid="{2FE3E094-F831-4B6A-8F68-958367A1890E}" name="WP_4" dataDxfId="35"/>
-    <tableColumn id="51" xr3:uid="{FDA92DA7-3473-43EC-9CF7-2973FA9CC4D4}" name="WP_4_unit" dataDxfId="34"/>
-    <tableColumn id="58" xr3:uid="{BE460051-3822-4F7B-9128-B9FF3E679D50}" name="initial_NO3_4" dataDxfId="33"/>
-    <tableColumn id="37" xr3:uid="{8064862C-F8DC-4543-B5CF-D282DD564B1D}" name="initial_NO3_4_unit" dataDxfId="32"/>
-    <tableColumn id="59" xr3:uid="{17C5A0C3-B5F4-4AAB-876C-FC876098B9C8}" name="initial_NH4_4" dataDxfId="31"/>
-    <tableColumn id="38" xr3:uid="{251884D5-BA16-4F6E-89D1-06011C0ABD02}" name="initial_NH4_4_unit" dataDxfId="30"/>
+    <tableColumn id="50" xr3:uid="{D1D16E63-48A7-4CF1-950A-55FD748CC035}" name="FC_4_unit" dataDxfId="21"/>
+    <tableColumn id="36" xr3:uid="{2FE3E094-F831-4B6A-8F68-958367A1890E}" name="WP_4" dataDxfId="20"/>
+    <tableColumn id="51" xr3:uid="{FDA92DA7-3473-43EC-9CF7-2973FA9CC4D4}" name="WP_4_unit" dataDxfId="19"/>
+    <tableColumn id="58" xr3:uid="{BE460051-3822-4F7B-9128-B9FF3E679D50}" name="initial_NO3_4" dataDxfId="18"/>
+    <tableColumn id="37" xr3:uid="{8064862C-F8DC-4543-B5CF-D282DD564B1D}" name="initial_NO3_4_unit" dataDxfId="17"/>
+    <tableColumn id="59" xr3:uid="{17C5A0C3-B5F4-4AAB-876C-FC876098B9C8}" name="initial_NH4_4" dataDxfId="16"/>
+    <tableColumn id="38" xr3:uid="{251884D5-BA16-4F6E-89D1-06011C0ABD02}" name="initial_NH4_4_unit" dataDxfId="15"/>
     <tableColumn id="46" xr3:uid="{5545ADBB-3E57-4FCE-9979-330500D810A6}" name="thickness_5"/>
     <tableColumn id="49" xr3:uid="{28F4610E-A232-42D7-866E-B72AB5FC38D8}" name="%_sand_5"/>
     <tableColumn id="60" xr3:uid="{9557F7B0-0944-4CA4-8B86-630B4073480C}" name="%_clay_5"/>
     <tableColumn id="61" xr3:uid="{6977D0A0-E571-46FB-8186-DF22D992C4B6}" name="BD_5"/>
     <tableColumn id="62" xr3:uid="{762BF513-B3A9-4714-B788-A74D32CD414B}" name="SOC_5"/>
     <tableColumn id="63" xr3:uid="{F840DA58-F957-445A-8704-4823DC13AEC7}" name="FC_5"/>
-    <tableColumn id="64" xr3:uid="{47AF2E86-82B6-4018-9B34-1B9AA21CC4AF}" name="FC_5_unit" dataDxfId="29"/>
+    <tableColumn id="64" xr3:uid="{47AF2E86-82B6-4018-9B34-1B9AA21CC4AF}" name="FC_5_unit" dataDxfId="14"/>
     <tableColumn id="65" xr3:uid="{73133DDD-77CC-4B8F-AF63-0B5537B95DE3}" name="WP_5"/>
-    <tableColumn id="66" xr3:uid="{7CB1FDF0-326D-4446-9AAC-1DB26A38AAB4}" name="WP_5_unit" dataDxfId="28"/>
+    <tableColumn id="66" xr3:uid="{7CB1FDF0-326D-4446-9AAC-1DB26A38AAB4}" name="WP_5_unit" dataDxfId="13"/>
     <tableColumn id="67" xr3:uid="{AF697735-FE14-47A1-8029-532D47D2E5C7}" name="initial_NO3_5"/>
-    <tableColumn id="68" xr3:uid="{B9420E91-6BD4-467A-B4C2-A6E2DEAE7AC0}" name="initial_NO3_5_unit" dataDxfId="27"/>
-    <tableColumn id="69" xr3:uid="{FF6305CB-A38F-4242-9850-7966AD42A38B}" name="initial_NH4_5" dataDxfId="26"/>
-    <tableColumn id="70" xr3:uid="{B5EFBF0D-28C6-43EC-8EBE-8FDCF2F3F407}" name="initial_NH4_5_unit" dataDxfId="25"/>
+    <tableColumn id="68" xr3:uid="{B9420E91-6BD4-467A-B4C2-A6E2DEAE7AC0}" name="initial_NO3_5_unit" dataDxfId="12"/>
+    <tableColumn id="69" xr3:uid="{FF6305CB-A38F-4242-9850-7966AD42A38B}" name="initial_NH4_5" dataDxfId="11"/>
+    <tableColumn id="70" xr3:uid="{B5EFBF0D-28C6-43EC-8EBE-8FDCF2F3F407}" name="initial_NH4_5_unit" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}" name="Table5" displayName="Table5" ref="A1:D109" totalsRowShown="0" headerRowBorderDxfId="24" tableBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}" name="Table5" displayName="Table5" ref="A1:D109" totalsRowShown="0" headerRowBorderDxfId="54" tableBorderDxfId="53">
   <autoFilter ref="A1:D109" xr:uid="{16C387FE-1D31-45D4-9107-29718893990C}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9BCD565A-9AEA-41E2-A4E9-5770EC475FD6}" name="station_name" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{2FFE488A-7A94-4C6D-BFBF-9D19F7354A7D}" name="latitude" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{7A348C5F-5ECA-4DC4-9498-87CB7828B623}" name="PET_calculation" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{528CFAC7-D6A1-4BF3-A218-92AEE6E73C93}" name="average_windspeed" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{9BCD565A-9AEA-41E2-A4E9-5770EC475FD6}" name="station_name" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{2FFE488A-7A94-4C6D-BFBF-9D19F7354A7D}" name="latitude" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{7A348C5F-5ECA-4DC4-9498-87CB7828B623}" name="PET_calculation" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{528CFAC7-D6A1-4BF3-A218-92AEE6E73C93}" name="average_windspeed" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}" name="Table8" displayName="Table8" ref="A2:J100" totalsRowShown="0" headerRowBorderDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}" name="Table8" displayName="Table8" ref="A2:J100" totalsRowShown="0" headerRowBorderDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="A2:J100" xr:uid="{0F5B8E89-2F05-4CC0-ACA9-79A38A5A9857}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{524AE2E3-B113-41B0-849D-8331462FB910}" name="usm_name" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{524AE2E3-B113-41B0-849D-8331462FB910}" name="usm_name" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{C58B90D4-B75A-409B-9D58-E09932ABF65C}" name="simulation_start"/>
-    <tableColumn id="3" xr3:uid="{DDB99A97-7CAB-4C4A-87B0-F44791A69661}" name="simulation_end" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{CA3AF775-2448-4D7D-9193-B5BBEE39AD09}" name="management_file_name" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{DDB99A97-7CAB-4C4A-87B0-F44791A69661}" name="simulation_end" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{CA3AF775-2448-4D7D-9193-B5BBEE39AD09}" name="management_file_name" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{C4CB74A7-2660-4D67-9D08-D7802D112D6D}" name="soil_profile_name"/>
     <tableColumn id="6" xr3:uid="{EE8564A9-D685-42B6-914D-B5F77F840B11}" name="weather_station_name"/>
     <tableColumn id="7" xr3:uid="{DF70C6E4-2795-4D3D-B86B-8B48BE8FB3E1}" name="plant_file"/>
-    <tableColumn id="8" xr3:uid="{B3D6750F-E334-4A3F-A048-BA40F1D2EC0C}" name="cultivar_code" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{B3D6750F-E334-4A3F-A048-BA40F1D2EC0C}" name="cultivar_code" dataDxfId="4"/>
     <tableColumn id="9" xr3:uid="{BDB57316-D9C6-4EE3-821F-F5561E0078D9}" name="first_year"/>
-    <tableColumn id="10" xr3:uid="{733885B2-6768-4BD5-9F65-4E7F4F6262F5}" name="last_year" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{733885B2-6768-4BD5-9F65-4E7F4F6262F5}" name="last_year" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}" name="Table10" displayName="Table10" ref="A1:F30" totalsRowShown="0" headerRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}" name="Table10" displayName="Table10" ref="A1:F30" totalsRowShown="0" headerRowBorderDxfId="2">
   <autoFilter ref="A1:F30" xr:uid="{16A01ECA-7371-41CC-818F-9452134FC132}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{F945B708-1D60-4D2B-99F2-60E35ECBDB15}" name="usm_name" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{F945B708-1D60-4D2B-99F2-60E35ECBDB15}" name="usm_name" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{A5156817-2D3F-4E14-AC57-75BA66E12293}" name="year"/>
     <tableColumn id="3" xr3:uid="{173E3383-07EB-425D-884F-01E4ECFF4626}" name="month"/>
-    <tableColumn id="4" xr3:uid="{786A5374-97E3-4942-B27A-E7E524EC0BA1}" name="day" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{786A5374-97E3-4942-B27A-E7E524EC0BA1}" name="day" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{B9B2B184-EF64-48EF-B50B-8E24249DFDCC}" name="variable 1"/>
     <tableColumn id="7" xr3:uid="{ED0F5D28-DB43-4C9B-ADB2-1706AC6D61F9}" name="variable 2"/>
   </tableColumns>
@@ -2088,7 +2142,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:AT100"/>
+  <dimension ref="A1:AX100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" style="5" customWidth="1"/>
@@ -2139,63 +2193,67 @@
     <col min="46" max="46" width="18.21875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.3">
-      <c r="C1" s="51" t="s">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C1" s="55" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="52" t="s">
+      <c r="D1" s="55"/>
+      <c r="E1" s="56" t="s">
         <v>63</v>
       </c>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="54" t="s">
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="53" t="s">
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
-      <c r="O1" s="53"/>
-      <c r="P1" s="55" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="55"/>
-      <c r="Z1" s="55"/>
-      <c r="AA1" s="55"/>
-      <c r="AB1" s="55"/>
-      <c r="AC1" s="55"/>
-      <c r="AD1" s="55"/>
-      <c r="AE1" s="55"/>
-      <c r="AF1" s="55"/>
-      <c r="AG1" s="55"/>
-      <c r="AH1" s="55"/>
-      <c r="AI1" s="55"/>
-      <c r="AJ1" s="55"/>
-      <c r="AK1" s="55"/>
-      <c r="AL1" s="55"/>
-      <c r="AM1" s="55"/>
-      <c r="AN1" s="55"/>
-      <c r="AO1" s="55"/>
-      <c r="AP1" s="55"/>
-      <c r="AQ1" s="55"/>
-      <c r="AR1" s="55"/>
-      <c r="AS1" s="55"/>
-      <c r="AT1" s="55"/>
-    </row>
-    <row r="2" spans="1:46" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="69" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="72"/>
+      <c r="AW1" s="70" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:50" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
         <v>52</v>
       </c>
@@ -2242,500 +2300,901 @@
         <v>62</v>
       </c>
       <c r="P2" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="R2" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="S2" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="T2" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="U2" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="V2" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="W2" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="V2" s="11" t="s">
+      <c r="X2" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="Y2" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="X2" s="11" t="s">
+      <c r="Z2" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="AA2" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="Z2" s="11" t="s">
+      <c r="AB2" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="AA2" s="11" t="s">
+      <c r="AC2" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="AB2" s="11" t="s">
+      <c r="AD2" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="AC2" s="11" t="s">
+      <c r="AE2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="AD2" s="11" t="s">
+      <c r="AF2" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="AE2" s="11" t="s">
+      <c r="AG2" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="AF2" s="11" t="s">
+      <c r="AH2" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="AG2" s="11" t="s">
+      <c r="AI2" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="AH2" s="11" t="s">
+      <c r="AJ2" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="AI2" s="11" t="s">
+      <c r="AK2" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="AJ2" s="11" t="s">
+      <c r="AL2" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="AK2" s="11" t="s">
+      <c r="AM2" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="AL2" s="11" t="s">
+      <c r="AN2" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="AM2" s="11" t="s">
+      <c r="AO2" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="AN2" s="11" t="s">
+      <c r="AP2" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="AO2" s="11" t="s">
+      <c r="AQ2" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="AP2" s="11" t="s">
+      <c r="AR2" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="AQ2" s="11" t="s">
+      <c r="AS2" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="AR2" s="11" t="s">
+      <c r="AT2" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="AS2" s="11" t="s">
+      <c r="AU2" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="AT2" s="11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.3">
-      <c r="E3" s="67"/>
+      <c r="AV2" s="71" t="s">
+        <v>170</v>
+      </c>
+      <c r="AW2" s="73" t="s">
+        <v>169</v>
+      </c>
+      <c r="AX2" s="73" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="E3" s="54"/>
       <c r="M3" s="38"/>
       <c r="N3" s="38"/>
+      <c r="P3" s="74"/>
+      <c r="Q3" s="68"/>
       <c r="AT3"/>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M4" s="38"/>
       <c r="N4" s="38"/>
-    </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P4" s="74"/>
+      <c r="Q4" s="68"/>
+      <c r="AT4"/>
+      <c r="AV4" s="68"/>
+    </row>
+    <row r="5" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M5" s="38"/>
       <c r="N5" s="38"/>
-    </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P5" s="74"/>
+      <c r="Q5" s="68"/>
+      <c r="AT5"/>
+      <c r="AV5" s="68"/>
+    </row>
+    <row r="6" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M6" s="38"/>
       <c r="N6" s="38"/>
-    </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P6" s="74"/>
+      <c r="Q6" s="68"/>
+      <c r="AT6"/>
+      <c r="AV6" s="68"/>
+    </row>
+    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M7" s="38"/>
       <c r="N7" s="38"/>
-    </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P7" s="74"/>
+      <c r="Q7" s="68"/>
+      <c r="AT7"/>
+      <c r="AV7" s="68"/>
+    </row>
+    <row r="8" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M8" s="38"/>
       <c r="N8" s="38"/>
-    </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P8" s="74"/>
+      <c r="Q8" s="68"/>
+      <c r="AT8"/>
+      <c r="AV8" s="68"/>
+    </row>
+    <row r="9" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M9" s="38"/>
       <c r="N9" s="38"/>
-    </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P9" s="74"/>
+      <c r="Q9" s="68"/>
+      <c r="AT9"/>
+      <c r="AV9" s="68"/>
+    </row>
+    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M10" s="38"/>
       <c r="N10" s="38"/>
-    </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P10" s="74"/>
+      <c r="Q10" s="68"/>
+      <c r="AT10"/>
+      <c r="AV10" s="68"/>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M11" s="38"/>
       <c r="N11" s="38"/>
-    </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P11" s="74"/>
+      <c r="Q11" s="68"/>
+      <c r="AT11"/>
+      <c r="AV11" s="68"/>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M12" s="38"/>
       <c r="N12" s="38"/>
-    </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P12" s="74"/>
+      <c r="Q12" s="68"/>
+      <c r="AT12"/>
+      <c r="AV12" s="68"/>
+    </row>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M13" s="38"/>
       <c r="N13" s="38"/>
-    </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P13" s="74"/>
+      <c r="Q13" s="68"/>
+      <c r="AT13"/>
+      <c r="AV13" s="68"/>
+    </row>
+    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M14" s="38"/>
       <c r="N14" s="38"/>
-    </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P14" s="74"/>
+      <c r="Q14" s="68"/>
+      <c r="AT14"/>
+      <c r="AV14" s="68"/>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M15" s="38"/>
       <c r="N15" s="38"/>
-    </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.3">
+      <c r="P15" s="74"/>
+      <c r="Q15" s="68"/>
+      <c r="AT15"/>
+      <c r="AV15" s="68"/>
+    </row>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
       <c r="M16" s="38"/>
       <c r="N16" s="38"/>
-    </row>
-    <row r="17" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P16" s="74"/>
+      <c r="Q16" s="68"/>
+      <c r="AT16"/>
+      <c r="AV16" s="68"/>
+    </row>
+    <row r="17" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M17" s="38"/>
       <c r="N17" s="38"/>
-    </row>
-    <row r="18" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P17" s="74"/>
+      <c r="Q17" s="68"/>
+      <c r="AT17"/>
+      <c r="AV17" s="68"/>
+    </row>
+    <row r="18" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M18" s="38"/>
       <c r="N18" s="38"/>
-    </row>
-    <row r="19" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P18" s="74"/>
+      <c r="Q18" s="68"/>
+      <c r="AT18"/>
+      <c r="AV18" s="68"/>
+    </row>
+    <row r="19" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M19" s="38"/>
       <c r="N19" s="38"/>
-    </row>
-    <row r="20" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P19" s="74"/>
+      <c r="Q19" s="68"/>
+      <c r="AT19"/>
+      <c r="AV19" s="68"/>
+    </row>
+    <row r="20" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M20" s="38"/>
       <c r="N20" s="38"/>
-    </row>
-    <row r="21" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P20" s="74"/>
+      <c r="Q20" s="68"/>
+      <c r="AT20"/>
+      <c r="AV20" s="68"/>
+    </row>
+    <row r="21" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M21" s="38"/>
       <c r="N21" s="38"/>
-    </row>
-    <row r="22" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P21" s="74"/>
+      <c r="Q21" s="68"/>
+      <c r="AT21"/>
+      <c r="AV21" s="68"/>
+    </row>
+    <row r="22" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M22" s="38"/>
       <c r="N22" s="38"/>
-    </row>
-    <row r="23" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P22" s="74"/>
+      <c r="Q22" s="68"/>
+      <c r="AT22"/>
+      <c r="AV22" s="68"/>
+    </row>
+    <row r="23" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M23" s="38"/>
       <c r="N23" s="38"/>
-    </row>
-    <row r="24" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P23" s="74"/>
+      <c r="Q23" s="68"/>
+      <c r="AT23"/>
+      <c r="AV23" s="68"/>
+    </row>
+    <row r="24" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M24" s="38"/>
       <c r="N24" s="38"/>
-    </row>
-    <row r="25" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P24" s="74"/>
+      <c r="Q24" s="68"/>
+      <c r="AT24"/>
+      <c r="AV24" s="68"/>
+    </row>
+    <row r="25" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M25" s="38"/>
       <c r="N25" s="38"/>
-    </row>
-    <row r="26" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P25" s="74"/>
+      <c r="Q25" s="68"/>
+      <c r="AT25"/>
+      <c r="AV25" s="68"/>
+    </row>
+    <row r="26" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M26" s="38"/>
       <c r="N26" s="38"/>
-    </row>
-    <row r="27" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P26" s="74"/>
+      <c r="Q26" s="68"/>
+      <c r="AT26"/>
+      <c r="AV26" s="68"/>
+    </row>
+    <row r="27" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M27" s="38"/>
       <c r="N27" s="38"/>
-    </row>
-    <row r="28" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P27" s="74"/>
+      <c r="Q27" s="68"/>
+      <c r="AT27"/>
+      <c r="AV27" s="68"/>
+    </row>
+    <row r="28" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M28" s="38"/>
       <c r="N28" s="38"/>
-    </row>
-    <row r="29" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P28" s="74"/>
+      <c r="Q28" s="68"/>
+      <c r="AT28"/>
+      <c r="AV28" s="68"/>
+    </row>
+    <row r="29" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M29" s="38"/>
       <c r="N29" s="38"/>
-    </row>
-    <row r="30" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P29" s="74"/>
+      <c r="Q29" s="68"/>
+      <c r="AT29"/>
+      <c r="AV29" s="68"/>
+    </row>
+    <row r="30" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M30" s="38"/>
       <c r="N30" s="38"/>
-    </row>
-    <row r="31" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P30" s="74"/>
+      <c r="Q30" s="68"/>
+      <c r="AT30"/>
+      <c r="AV30" s="68"/>
+    </row>
+    <row r="31" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M31" s="38"/>
       <c r="N31" s="38"/>
-    </row>
-    <row r="32" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P31" s="74"/>
+      <c r="Q31" s="68"/>
+      <c r="AT31"/>
+      <c r="AV31" s="68"/>
+    </row>
+    <row r="32" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M32" s="38"/>
       <c r="N32" s="38"/>
-    </row>
-    <row r="33" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P32" s="74"/>
+      <c r="Q32" s="68"/>
+      <c r="AT32"/>
+      <c r="AV32" s="68"/>
+    </row>
+    <row r="33" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M33" s="38"/>
       <c r="N33" s="38"/>
-    </row>
-    <row r="34" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P33" s="74"/>
+      <c r="Q33" s="68"/>
+      <c r="AT33"/>
+      <c r="AV33" s="68"/>
+    </row>
+    <row r="34" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M34" s="38"/>
       <c r="N34" s="38"/>
-    </row>
-    <row r="35" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P34" s="74"/>
+      <c r="Q34" s="68"/>
+      <c r="AT34"/>
+      <c r="AV34" s="68"/>
+    </row>
+    <row r="35" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M35" s="38"/>
       <c r="N35" s="38"/>
-    </row>
-    <row r="36" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P35" s="74"/>
+      <c r="Q35" s="68"/>
+      <c r="AT35"/>
+      <c r="AV35" s="68"/>
+    </row>
+    <row r="36" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M36" s="38"/>
       <c r="N36" s="38"/>
-    </row>
-    <row r="37" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P36" s="74"/>
+      <c r="Q36" s="68"/>
+      <c r="AT36"/>
+      <c r="AV36" s="68"/>
+    </row>
+    <row r="37" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M37" s="38"/>
       <c r="N37" s="38"/>
-    </row>
-    <row r="38" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P37" s="74"/>
+      <c r="Q37" s="68"/>
+      <c r="AT37"/>
+      <c r="AV37" s="68"/>
+    </row>
+    <row r="38" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M38" s="38"/>
       <c r="N38" s="38"/>
-    </row>
-    <row r="39" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P38" s="74"/>
+      <c r="Q38" s="68"/>
+      <c r="AT38"/>
+      <c r="AV38" s="68"/>
+    </row>
+    <row r="39" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M39" s="38"/>
       <c r="N39" s="38"/>
-    </row>
-    <row r="40" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P39" s="74"/>
+      <c r="Q39" s="68"/>
+      <c r="AT39"/>
+      <c r="AV39" s="68"/>
+    </row>
+    <row r="40" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M40" s="38"/>
       <c r="N40" s="38"/>
-    </row>
-    <row r="41" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P40" s="74"/>
+      <c r="Q40" s="68"/>
+      <c r="AT40"/>
+      <c r="AV40" s="68"/>
+    </row>
+    <row r="41" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M41" s="38"/>
       <c r="N41" s="38"/>
-    </row>
-    <row r="42" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P41" s="74"/>
+      <c r="Q41" s="68"/>
+      <c r="AT41"/>
+      <c r="AV41" s="68"/>
+    </row>
+    <row r="42" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M42" s="38"/>
       <c r="N42" s="38"/>
-    </row>
-    <row r="43" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P42" s="74"/>
+      <c r="Q42" s="68"/>
+      <c r="AT42"/>
+      <c r="AV42" s="68"/>
+    </row>
+    <row r="43" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M43" s="38"/>
       <c r="N43" s="38"/>
-    </row>
-    <row r="44" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P43" s="74"/>
+      <c r="Q43" s="68"/>
+      <c r="AT43"/>
+      <c r="AV43" s="68"/>
+    </row>
+    <row r="44" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M44" s="38"/>
       <c r="N44" s="38"/>
-    </row>
-    <row r="45" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P44" s="74"/>
+      <c r="Q44" s="68"/>
+      <c r="AT44"/>
+      <c r="AV44" s="68"/>
+    </row>
+    <row r="45" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M45" s="38"/>
       <c r="N45" s="38"/>
-    </row>
-    <row r="46" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P45" s="74"/>
+      <c r="Q45" s="68"/>
+      <c r="AT45"/>
+      <c r="AV45" s="68"/>
+    </row>
+    <row r="46" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M46" s="38"/>
       <c r="N46" s="38"/>
-    </row>
-    <row r="47" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P46" s="74"/>
+      <c r="Q46" s="68"/>
+      <c r="AT46"/>
+      <c r="AV46" s="68"/>
+    </row>
+    <row r="47" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M47" s="38"/>
       <c r="N47" s="38"/>
-    </row>
-    <row r="48" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P47" s="74"/>
+      <c r="Q47" s="68"/>
+      <c r="AT47"/>
+      <c r="AV47" s="68"/>
+    </row>
+    <row r="48" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M48" s="38"/>
       <c r="N48" s="38"/>
-    </row>
-    <row r="49" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P48" s="74"/>
+      <c r="Q48" s="68"/>
+      <c r="AT48"/>
+      <c r="AV48" s="68"/>
+    </row>
+    <row r="49" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M49" s="38"/>
       <c r="N49" s="38"/>
-    </row>
-    <row r="50" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P49" s="74"/>
+      <c r="Q49" s="68"/>
+      <c r="AT49"/>
+      <c r="AV49" s="68"/>
+    </row>
+    <row r="50" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M50" s="38"/>
       <c r="N50" s="38"/>
-    </row>
-    <row r="51" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P50" s="74"/>
+      <c r="Q50" s="68"/>
+      <c r="AT50"/>
+      <c r="AV50" s="68"/>
+    </row>
+    <row r="51" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M51" s="38"/>
       <c r="N51" s="38"/>
-    </row>
-    <row r="52" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P51" s="74"/>
+      <c r="Q51" s="68"/>
+      <c r="AT51"/>
+      <c r="AV51" s="68"/>
+    </row>
+    <row r="52" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M52" s="38"/>
       <c r="N52" s="38"/>
-    </row>
-    <row r="53" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P52" s="74"/>
+      <c r="Q52" s="68"/>
+      <c r="AT52"/>
+      <c r="AV52" s="68"/>
+    </row>
+    <row r="53" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M53" s="38"/>
       <c r="N53" s="38"/>
-    </row>
-    <row r="54" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P53" s="74"/>
+      <c r="Q53" s="68"/>
+      <c r="AT53"/>
+      <c r="AV53" s="68"/>
+    </row>
+    <row r="54" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M54" s="38"/>
       <c r="N54" s="38"/>
-    </row>
-    <row r="55" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P54" s="74"/>
+      <c r="Q54" s="68"/>
+      <c r="AT54"/>
+      <c r="AV54" s="68"/>
+    </row>
+    <row r="55" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M55" s="38"/>
       <c r="N55" s="38"/>
-    </row>
-    <row r="56" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P55" s="74"/>
+      <c r="Q55" s="68"/>
+      <c r="AT55"/>
+      <c r="AV55" s="68"/>
+    </row>
+    <row r="56" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M56" s="38"/>
       <c r="N56" s="38"/>
-    </row>
-    <row r="57" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P56" s="74"/>
+      <c r="Q56" s="68"/>
+      <c r="AT56"/>
+      <c r="AV56" s="68"/>
+    </row>
+    <row r="57" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M57" s="38"/>
       <c r="N57" s="38"/>
-    </row>
-    <row r="58" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P57" s="74"/>
+      <c r="Q57" s="68"/>
+      <c r="AT57"/>
+      <c r="AV57" s="68"/>
+    </row>
+    <row r="58" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M58" s="38"/>
       <c r="N58" s="38"/>
-    </row>
-    <row r="59" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P58" s="74"/>
+      <c r="Q58" s="68"/>
+      <c r="AT58"/>
+      <c r="AV58" s="68"/>
+    </row>
+    <row r="59" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M59" s="38"/>
       <c r="N59" s="38"/>
-    </row>
-    <row r="60" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P59" s="74"/>
+      <c r="Q59" s="68"/>
+      <c r="AT59"/>
+      <c r="AV59" s="68"/>
+    </row>
+    <row r="60" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M60" s="38"/>
       <c r="N60" s="38"/>
-    </row>
-    <row r="61" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P60" s="74"/>
+      <c r="Q60" s="68"/>
+      <c r="AT60"/>
+      <c r="AV60" s="68"/>
+    </row>
+    <row r="61" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M61" s="38"/>
       <c r="N61" s="38"/>
-    </row>
-    <row r="62" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P61" s="74"/>
+      <c r="Q61" s="68"/>
+      <c r="AT61"/>
+      <c r="AV61" s="68"/>
+    </row>
+    <row r="62" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M62" s="38"/>
       <c r="N62" s="38"/>
-    </row>
-    <row r="63" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P62" s="74"/>
+      <c r="Q62" s="68"/>
+      <c r="AT62"/>
+      <c r="AV62" s="68"/>
+    </row>
+    <row r="63" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M63" s="38"/>
       <c r="N63" s="38"/>
-    </row>
-    <row r="64" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P63" s="74"/>
+      <c r="Q63" s="68"/>
+      <c r="AT63"/>
+      <c r="AV63" s="68"/>
+    </row>
+    <row r="64" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M64" s="38"/>
       <c r="N64" s="38"/>
-    </row>
-    <row r="65" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P64" s="74"/>
+      <c r="Q64" s="68"/>
+      <c r="AT64"/>
+      <c r="AV64" s="68"/>
+    </row>
+    <row r="65" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M65" s="38"/>
       <c r="N65" s="38"/>
-    </row>
-    <row r="66" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P65" s="74"/>
+      <c r="Q65" s="68"/>
+      <c r="AT65"/>
+      <c r="AV65" s="68"/>
+    </row>
+    <row r="66" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M66" s="38"/>
       <c r="N66" s="38"/>
-    </row>
-    <row r="67" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P66" s="74"/>
+      <c r="Q66" s="68"/>
+      <c r="AT66"/>
+      <c r="AV66" s="68"/>
+    </row>
+    <row r="67" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M67" s="38"/>
       <c r="N67" s="38"/>
-    </row>
-    <row r="68" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P67" s="74"/>
+      <c r="Q67" s="68"/>
+      <c r="AT67"/>
+      <c r="AV67" s="68"/>
+    </row>
+    <row r="68" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M68" s="38"/>
       <c r="N68" s="38"/>
-    </row>
-    <row r="69" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P68" s="74"/>
+      <c r="Q68" s="68"/>
+      <c r="AT68"/>
+      <c r="AV68" s="68"/>
+    </row>
+    <row r="69" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M69" s="38"/>
       <c r="N69" s="38"/>
-    </row>
-    <row r="70" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P69" s="74"/>
+      <c r="Q69" s="68"/>
+      <c r="AT69"/>
+      <c r="AV69" s="68"/>
+    </row>
+    <row r="70" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M70" s="38"/>
       <c r="N70" s="38"/>
-    </row>
-    <row r="71" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P70" s="74"/>
+      <c r="Q70" s="68"/>
+      <c r="AT70"/>
+      <c r="AV70" s="68"/>
+    </row>
+    <row r="71" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M71" s="38"/>
       <c r="N71" s="38"/>
-    </row>
-    <row r="72" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P71" s="74"/>
+      <c r="Q71" s="68"/>
+      <c r="AT71"/>
+      <c r="AV71" s="68"/>
+    </row>
+    <row r="72" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M72" s="38"/>
       <c r="N72" s="38"/>
-    </row>
-    <row r="73" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P72" s="74"/>
+      <c r="Q72" s="68"/>
+      <c r="AT72"/>
+      <c r="AV72" s="68"/>
+    </row>
+    <row r="73" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M73" s="38"/>
       <c r="N73" s="38"/>
-    </row>
-    <row r="74" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P73" s="74"/>
+      <c r="Q73" s="68"/>
+      <c r="AT73"/>
+      <c r="AV73" s="68"/>
+    </row>
+    <row r="74" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M74" s="38"/>
       <c r="N74" s="38"/>
-    </row>
-    <row r="75" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P74" s="74"/>
+      <c r="Q74" s="68"/>
+      <c r="AT74"/>
+      <c r="AV74" s="68"/>
+    </row>
+    <row r="75" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M75" s="38"/>
       <c r="N75" s="38"/>
-    </row>
-    <row r="76" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P75" s="74"/>
+      <c r="Q75" s="68"/>
+      <c r="AT75"/>
+      <c r="AV75" s="68"/>
+    </row>
+    <row r="76" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M76" s="38"/>
       <c r="N76" s="38"/>
-    </row>
-    <row r="77" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P76" s="74"/>
+      <c r="Q76" s="68"/>
+      <c r="AT76"/>
+      <c r="AV76" s="68"/>
+    </row>
+    <row r="77" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M77" s="38"/>
       <c r="N77" s="38"/>
-    </row>
-    <row r="78" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P77" s="74"/>
+      <c r="Q77" s="68"/>
+      <c r="AT77"/>
+      <c r="AV77" s="68"/>
+    </row>
+    <row r="78" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M78" s="38"/>
       <c r="N78" s="38"/>
-    </row>
-    <row r="79" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P78" s="74"/>
+      <c r="Q78" s="68"/>
+      <c r="AT78"/>
+      <c r="AV78" s="68"/>
+    </row>
+    <row r="79" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M79" s="38"/>
       <c r="N79" s="38"/>
-    </row>
-    <row r="80" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P79" s="74"/>
+      <c r="Q79" s="68"/>
+      <c r="AT79"/>
+      <c r="AV79" s="68"/>
+    </row>
+    <row r="80" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M80" s="38"/>
       <c r="N80" s="38"/>
-    </row>
-    <row r="81" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P80" s="74"/>
+      <c r="Q80" s="68"/>
+      <c r="AT80"/>
+      <c r="AV80" s="68"/>
+    </row>
+    <row r="81" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M81" s="38"/>
       <c r="N81" s="38"/>
-    </row>
-    <row r="82" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P81" s="74"/>
+      <c r="Q81" s="68"/>
+      <c r="AT81"/>
+      <c r="AV81" s="68"/>
+    </row>
+    <row r="82" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M82" s="38"/>
       <c r="N82" s="38"/>
-    </row>
-    <row r="83" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P82" s="74"/>
+      <c r="Q82" s="68"/>
+      <c r="AT82"/>
+      <c r="AV82" s="68"/>
+    </row>
+    <row r="83" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M83" s="38"/>
       <c r="N83" s="38"/>
-    </row>
-    <row r="84" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P83" s="74"/>
+      <c r="Q83" s="68"/>
+      <c r="AT83"/>
+      <c r="AV83" s="68"/>
+    </row>
+    <row r="84" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M84" s="38"/>
       <c r="N84" s="38"/>
-    </row>
-    <row r="85" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P84" s="74"/>
+      <c r="Q84" s="68"/>
+      <c r="AT84"/>
+      <c r="AV84" s="68"/>
+    </row>
+    <row r="85" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M85" s="38"/>
       <c r="N85" s="38"/>
-    </row>
-    <row r="86" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P85" s="74"/>
+      <c r="Q85" s="68"/>
+      <c r="AT85"/>
+      <c r="AV85" s="68"/>
+    </row>
+    <row r="86" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M86" s="38"/>
       <c r="N86" s="38"/>
-    </row>
-    <row r="87" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P86" s="74"/>
+      <c r="Q86" s="68"/>
+      <c r="AT86"/>
+      <c r="AV86" s="68"/>
+    </row>
+    <row r="87" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M87" s="38"/>
       <c r="N87" s="38"/>
-    </row>
-    <row r="88" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P87" s="74"/>
+      <c r="Q87" s="68"/>
+      <c r="AT87"/>
+      <c r="AV87" s="68"/>
+    </row>
+    <row r="88" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M88" s="38"/>
       <c r="N88" s="38"/>
-    </row>
-    <row r="89" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P88" s="74"/>
+      <c r="Q88" s="68"/>
+      <c r="AT88"/>
+      <c r="AV88" s="68"/>
+    </row>
+    <row r="89" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M89" s="38"/>
       <c r="N89" s="38"/>
-    </row>
-    <row r="90" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P89" s="74"/>
+      <c r="Q89" s="68"/>
+      <c r="AT89"/>
+      <c r="AV89" s="68"/>
+    </row>
+    <row r="90" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M90" s="38"/>
       <c r="N90" s="38"/>
-    </row>
-    <row r="91" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P90" s="74"/>
+      <c r="Q90" s="68"/>
+      <c r="AT90"/>
+      <c r="AV90" s="68"/>
+    </row>
+    <row r="91" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M91" s="38"/>
       <c r="N91" s="38"/>
-    </row>
-    <row r="92" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P91" s="74"/>
+      <c r="Q91" s="68"/>
+      <c r="AT91"/>
+      <c r="AV91" s="68"/>
+    </row>
+    <row r="92" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M92" s="38"/>
       <c r="N92" s="38"/>
-    </row>
-    <row r="93" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P92" s="74"/>
+      <c r="Q92" s="68"/>
+      <c r="AT92"/>
+      <c r="AV92" s="68"/>
+    </row>
+    <row r="93" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M93" s="38"/>
       <c r="N93" s="38"/>
-    </row>
-    <row r="94" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P93" s="74"/>
+      <c r="Q93" s="68"/>
+      <c r="AT93"/>
+      <c r="AV93" s="68"/>
+    </row>
+    <row r="94" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M94" s="38"/>
       <c r="N94" s="38"/>
-    </row>
-    <row r="95" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P94" s="74"/>
+      <c r="Q94" s="68"/>
+      <c r="AT94"/>
+      <c r="AV94" s="68"/>
+    </row>
+    <row r="95" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M95" s="38"/>
       <c r="N95" s="38"/>
-    </row>
-    <row r="96" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P95" s="74"/>
+      <c r="Q95" s="68"/>
+      <c r="AT95"/>
+      <c r="AV95" s="68"/>
+    </row>
+    <row r="96" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M96" s="38"/>
       <c r="N96" s="38"/>
-    </row>
-    <row r="97" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P96" s="74"/>
+      <c r="Q96" s="68"/>
+      <c r="AT96"/>
+      <c r="AV96" s="68"/>
+    </row>
+    <row r="97" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M97" s="38"/>
       <c r="N97" s="38"/>
-    </row>
-    <row r="98" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P97" s="74"/>
+      <c r="Q97" s="68"/>
+      <c r="AT97"/>
+      <c r="AV97" s="68"/>
+    </row>
+    <row r="98" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M98" s="38"/>
       <c r="N98" s="38"/>
-    </row>
-    <row r="99" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P98" s="74"/>
+      <c r="Q98" s="68"/>
+      <c r="AT98"/>
+      <c r="AV98" s="68"/>
+    </row>
+    <row r="99" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M99" s="38"/>
       <c r="N99" s="38"/>
-    </row>
-    <row r="100" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="P99" s="74"/>
+      <c r="Q99" s="68"/>
+      <c r="AT99"/>
+      <c r="AV99" s="68"/>
+    </row>
+    <row r="100" spans="13:48" x14ac:dyDescent="0.3">
       <c r="M100" s="38"/>
       <c r="N100" s="38"/>
+      <c r="P100" s="74"/>
+      <c r="Q100" s="68"/>
+      <c r="AT100"/>
+      <c r="AV100" s="68"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="K1:O1"/>
     <mergeCell ref="H1:J1"/>
-    <mergeCell ref="P1:AT1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2744,7 +3203,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="fertilizer" prompt="select type" xr:uid="{B70B515A-9E4D-43A4-A403-3B52F4B6E7A5}">
           <x14:formula1>
             <xm:f>options!$C$2:$C$9</xm:f>
@@ -2756,6 +3215,12 @@
             <xm:f>options!$E$2:$E$3</xm:f>
           </x14:formula1>
           <xm:sqref>N3:N100</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="irrigation location" prompt="Indicate if irrigation applied aboveground (either above or below plant canopy) or belowground (i.e. drip). " xr:uid="{D1AF471D-DDE0-4230-AA87-8B03F8E0C30A}">
+          <x14:formula1>
+            <xm:f>options!$K$2:$K$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>P3:P100</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2797,85 +3262,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:71" x14ac:dyDescent="0.3">
-      <c r="B1" s="56" t="s">
+      <c r="B1" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
-      <c r="P1" s="56"/>
-      <c r="Q1" s="56"/>
-      <c r="R1" s="56"/>
-      <c r="S1" s="52" t="s">
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="T1" s="52"/>
-      <c r="U1" s="52"/>
-      <c r="V1" s="52"/>
-      <c r="W1" s="52"/>
-      <c r="X1" s="52"/>
-      <c r="Y1" s="52"/>
-      <c r="Z1" s="52"/>
-      <c r="AA1" s="52"/>
-      <c r="AB1" s="52"/>
-      <c r="AC1" s="52"/>
-      <c r="AD1" s="52"/>
-      <c r="AE1" s="52"/>
-      <c r="AF1" s="51" t="s">
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
+      <c r="W1" s="56"/>
+      <c r="X1" s="56"/>
+      <c r="Y1" s="56"/>
+      <c r="Z1" s="56"/>
+      <c r="AA1" s="56"/>
+      <c r="AB1" s="56"/>
+      <c r="AC1" s="56"/>
+      <c r="AD1" s="56"/>
+      <c r="AE1" s="56"/>
+      <c r="AF1" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="AG1" s="51"/>
-      <c r="AH1" s="51"/>
-      <c r="AI1" s="51"/>
-      <c r="AJ1" s="51"/>
-      <c r="AK1" s="51"/>
-      <c r="AL1" s="51"/>
-      <c r="AM1" s="51"/>
-      <c r="AN1" s="51"/>
-      <c r="AO1" s="51"/>
-      <c r="AP1" s="51"/>
-      <c r="AQ1" s="51"/>
-      <c r="AR1" s="51"/>
-      <c r="AS1" s="55" t="s">
+      <c r="AG1" s="55"/>
+      <c r="AH1" s="55"/>
+      <c r="AI1" s="55"/>
+      <c r="AJ1" s="55"/>
+      <c r="AK1" s="55"/>
+      <c r="AL1" s="55"/>
+      <c r="AM1" s="55"/>
+      <c r="AN1" s="55"/>
+      <c r="AO1" s="55"/>
+      <c r="AP1" s="55"/>
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="55"/>
+      <c r="AS1" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="AT1" s="55"/>
-      <c r="AU1" s="55"/>
-      <c r="AV1" s="55"/>
-      <c r="AW1" s="55"/>
-      <c r="AX1" s="55"/>
-      <c r="AY1" s="55"/>
-      <c r="AZ1" s="55"/>
-      <c r="BA1" s="55"/>
-      <c r="BB1" s="55"/>
-      <c r="BC1" s="55"/>
-      <c r="BD1" s="55"/>
-      <c r="BE1" s="57"/>
-      <c r="BF1" s="58" t="s">
-        <v>150</v>
-      </c>
-      <c r="BG1" s="58"/>
-      <c r="BH1" s="58"/>
-      <c r="BI1" s="58"/>
-      <c r="BJ1" s="58"/>
-      <c r="BK1" s="58"/>
-      <c r="BL1" s="58"/>
-      <c r="BM1" s="58"/>
-      <c r="BN1" s="58"/>
-      <c r="BO1" s="58"/>
-      <c r="BP1" s="58"/>
-      <c r="BQ1" s="58"/>
-      <c r="BR1" s="59"/>
+      <c r="AT1" s="59"/>
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="59"/>
+      <c r="AW1" s="59"/>
+      <c r="AX1" s="59"/>
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="59"/>
+      <c r="BA1" s="59"/>
+      <c r="BB1" s="59"/>
+      <c r="BC1" s="59"/>
+      <c r="BD1" s="59"/>
+      <c r="BE1" s="61"/>
+      <c r="BF1" s="62" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG1" s="62"/>
+      <c r="BH1" s="62"/>
+      <c r="BI1" s="62"/>
+      <c r="BJ1" s="62"/>
+      <c r="BK1" s="62"/>
+      <c r="BL1" s="62"/>
+      <c r="BM1" s="62"/>
+      <c r="BN1" s="62"/>
+      <c r="BO1" s="62"/>
+      <c r="BP1" s="62"/>
+      <c r="BQ1" s="62"/>
+      <c r="BR1" s="63"/>
     </row>
     <row r="2" spans="1:71" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
@@ -2888,7 +3353,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E2" s="27" t="s">
         <v>11</v>
@@ -2900,40 +3365,40 @@
         <v>13</v>
       </c>
       <c r="H2" s="27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I2" s="27" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="K2" s="27" t="s">
         <v>126</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>127</v>
       </c>
       <c r="L2" s="27" t="s">
         <v>43</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N2" s="27" t="s">
         <v>44</v>
       </c>
       <c r="O2" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P2" s="27" t="s">
         <v>15</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="R2" s="29" t="s">
         <v>16</v>
       </c>
       <c r="S2" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="T2" s="30" t="s">
         <v>18</v>
@@ -2954,25 +3419,25 @@
         <v>45</v>
       </c>
       <c r="Z2" s="24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>46</v>
       </c>
       <c r="AB2" s="24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC2" s="30" t="s">
         <v>23</v>
       </c>
       <c r="AD2" s="24" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AE2" s="31" t="s">
         <v>24</v>
       </c>
       <c r="AF2" s="25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG2" s="32" t="s">
         <v>25</v>
@@ -2993,25 +3458,25 @@
         <v>47</v>
       </c>
       <c r="AM2" s="34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AN2" s="32" t="s">
         <v>48</v>
       </c>
       <c r="AO2" s="34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AP2" s="32" t="s">
         <v>30</v>
       </c>
       <c r="AQ2" s="34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AR2" s="33" t="s">
         <v>31</v>
       </c>
       <c r="AS2" s="35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AT2" s="36" t="s">
         <v>32</v>
@@ -3032,64 +3497,64 @@
         <v>49</v>
       </c>
       <c r="AZ2" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="BA2" s="36" t="s">
         <v>50</v>
       </c>
       <c r="BB2" s="37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="BC2" s="36" t="s">
         <v>37</v>
       </c>
       <c r="BD2" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="BE2" s="36" t="s">
         <v>38</v>
       </c>
       <c r="BF2" s="44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="BG2" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="BH2" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="BH2" s="46" t="s">
+      <c r="BI2" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="BI2" s="46" t="s">
+      <c r="BJ2" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="BJ2" s="46" t="s">
+      <c r="BK2" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="BK2" s="46" t="s">
+      <c r="BL2" s="46" t="s">
         <v>155</v>
       </c>
-      <c r="BL2" s="46" t="s">
+      <c r="BM2" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="BM2" s="47" t="s">
+      <c r="BN2" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="BN2" s="46" t="s">
+      <c r="BO2" s="47" t="s">
         <v>158</v>
       </c>
-      <c r="BO2" s="47" t="s">
+      <c r="BP2" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="BP2" s="46" t="s">
+      <c r="BQ2" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="BQ2" s="47" t="s">
+      <c r="BR2" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="BR2" s="46" t="s">
+      <c r="BS2" s="48" t="s">
         <v>162</v>
-      </c>
-      <c r="BS2" s="48" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:71" x14ac:dyDescent="0.3">
@@ -6477,16 +6942,16 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C1"/>
-      <c r="D1" s="60" t="s">
+      <c r="D1" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="61"/>
-      <c r="I1" s="62" t="s">
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="67"/>
+      <c r="I1" s="64" t="s">
         <v>86</v>
       </c>
-      <c r="J1" s="63"/>
+      <c r="J1" s="65"/>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
@@ -7061,23 +7526,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>91</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D1" s="53" t="s">
         <v>164</v>
       </c>
-      <c r="D1" s="66" t="s">
+      <c r="E1" s="51" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="51" t="s">
         <v>165</v>
-      </c>
-      <c r="E1" s="64" t="s">
-        <v>167</v>
-      </c>
-      <c r="F1" s="64" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -7189,7 +7654,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA73EF4-F459-4FB8-999B-97CF29F368C2}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" customWidth="1"/>
@@ -7197,9 +7662,10 @@
     <col min="5" max="5" width="20.44140625" customWidth="1"/>
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="11" max="11" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>72</v>
       </c>
@@ -7210,13 +7676,16 @@
         <v>74</v>
       </c>
       <c r="G1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="K1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -7227,13 +7696,16 @@
         <v>75</v>
       </c>
       <c r="G2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+      <c r="K2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -7244,21 +7716,27 @@
         <v>76</v>
       </c>
       <c r="G3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+      <c r="K3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>70</v>
       </c>
       <c r="C4" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -7266,37 +7744,38 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="5">
+  <tableParts count="6">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>